<commit_message>
Add 'Take Over Time' sheet + chart: role share of the take by year
Compounds Athanase net returns (Sheet1) from an editable starting AUM into a
year-by-year AUM path (2006-2026), interpolates each role's headcount across
the AUM scenarios, and computes each role's % of the take (comp pool) per
year. Adds a native Excel line chart plus a stacked-area PNG. Shares sum to
100% each year; the CIO share compresses as investment roles expand.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K14qB8MpeJ8Pk8H1GeEUV4
</commit_message>
<xml_diff>
--- a/Performance_Fee_Framework.xlsx
+++ b/Performance_Fee_Framework.xlsx
@@ -7,7 +7,8 @@
   </bookViews>
   <sheets>
     <sheet name="Static" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Take Over Time" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="27">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -160,6 +161,33 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -222,7 +250,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -253,12 +281,56 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -378,6 +450,47 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="23" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="25" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -455,6 +568,510 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Role share of the take over time (%)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A8</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$8:$V$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$9:$V$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$10:$V$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$11:$V$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$12:$V$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A13</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$13:$V$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A14</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$14:$V$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A15</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$15:$V$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A16</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$16:$V$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A17</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$17:$V$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A18</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$18:$V$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A19</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$19:$V$19</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
+          <tx>
+            <strRef>
+              <f>'Take Over Time'!A20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take Over Time'!$B$6:$V$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take Over Time'!$B$20:$V$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% of take</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -479,6 +1096,33 @@
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9360000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -847,6 +1491,10 @@
           <t>Performance-fee rate (of profits)</t>
         </is>
       </c>
+      <c r="B5" s="59" t="n"/>
+      <c r="C5" s="59" t="n"/>
+      <c r="D5" s="59" t="n"/>
+      <c r="E5" s="60" t="n"/>
       <c r="F5" s="26" t="n">
         <v>0.2</v>
       </c>
@@ -857,6 +1505,10 @@
           <t>Firm take rate — share of perf-fee funding the comp pool</t>
         </is>
       </c>
+      <c r="B6" s="59" t="n"/>
+      <c r="C6" s="59" t="n"/>
+      <c r="D6" s="59" t="n"/>
+      <c r="E6" s="60" t="n"/>
       <c r="F6" s="26" t="n">
         <v>0.6</v>
       </c>
@@ -867,6 +1519,10 @@
           <t>AUM tier threshold (USD millions)</t>
         </is>
       </c>
+      <c r="B7" s="59" t="n"/>
+      <c r="C7" s="59" t="n"/>
+      <c r="D7" s="59" t="n"/>
+      <c r="E7" s="60" t="n"/>
       <c r="F7" s="27" t="n">
         <v>300</v>
       </c>
@@ -877,6 +1533,10 @@
           <t>Assumed gross return on AUM (drives the demo profit)</t>
         </is>
       </c>
+      <c r="B8" s="59" t="n"/>
+      <c r="C8" s="59" t="n"/>
+      <c r="D8" s="59" t="n"/>
+      <c r="E8" s="60" t="n"/>
       <c r="F8" s="26" t="n">
         <v>0.15</v>
       </c>
@@ -3347,8 +4007,8 @@
     <mergeCell ref="A94:M94"/>
     <mergeCell ref="A93:M93"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A97:M97"/>
     <mergeCell ref="A95:M95"/>
-    <mergeCell ref="A97:M97"/>
     <mergeCell ref="A92:M92"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A8:E8"/>
@@ -3361,6 +4021,1215 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="18" max="18"/>
+    <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="7" customWidth="1" min="20" max="20"/>
+    <col width="7" customWidth="1" min="21" max="21"/>
+    <col width="7" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="61" t="inlineStr">
+        <is>
+          <t>Each role's share of the take (comp pool), over time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="62" t="inlineStr">
+        <is>
+          <t>Share = role weight × headcount ÷ total weighted units. Headcount scales with the AUM path; % sums to 100% each year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="63" t="inlineStr">
+        <is>
+          <t>Starting AUM (USD m), compounded by Athanase net returns:</t>
+        </is>
+      </c>
+      <c r="D4" s="64" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="65" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B6" s="65" t="n">
+        <v>2006</v>
+      </c>
+      <c r="C6" s="65" t="n">
+        <v>2007</v>
+      </c>
+      <c r="D6" s="65" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E6" s="65" t="n">
+        <v>2009</v>
+      </c>
+      <c r="F6" s="65" t="n">
+        <v>2010</v>
+      </c>
+      <c r="G6" s="65" t="n">
+        <v>2011</v>
+      </c>
+      <c r="H6" s="65" t="n">
+        <v>2012</v>
+      </c>
+      <c r="I6" s="65" t="n">
+        <v>2013</v>
+      </c>
+      <c r="J6" s="65" t="n">
+        <v>2014</v>
+      </c>
+      <c r="K6" s="65" t="n">
+        <v>2015</v>
+      </c>
+      <c r="L6" s="65" t="n">
+        <v>2016</v>
+      </c>
+      <c r="M6" s="65" t="n">
+        <v>2017</v>
+      </c>
+      <c r="N6" s="65" t="n">
+        <v>2018</v>
+      </c>
+      <c r="O6" s="65" t="n">
+        <v>2019</v>
+      </c>
+      <c r="P6" s="65" t="n">
+        <v>2020</v>
+      </c>
+      <c r="Q6" s="65" t="n">
+        <v>2021</v>
+      </c>
+      <c r="R6" s="65" t="n">
+        <v>2022</v>
+      </c>
+      <c r="S6" s="65" t="n">
+        <v>2023</v>
+      </c>
+      <c r="T6" s="65" t="n">
+        <v>2024</v>
+      </c>
+      <c r="U6" s="65" t="n">
+        <v>2025</v>
+      </c>
+      <c r="V6" s="65" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="66" t="inlineStr">
+        <is>
+          <t>AUM (USD m)</t>
+        </is>
+      </c>
+      <c r="B7" s="67" t="n">
+        <v>162</v>
+      </c>
+      <c r="C7" s="67" t="n">
+        <v>149</v>
+      </c>
+      <c r="D7" s="67" t="n">
+        <v>88</v>
+      </c>
+      <c r="E7" s="67" t="n">
+        <v>159</v>
+      </c>
+      <c r="F7" s="67" t="n">
+        <v>205</v>
+      </c>
+      <c r="G7" s="67" t="n">
+        <v>201</v>
+      </c>
+      <c r="H7" s="67" t="n">
+        <v>211</v>
+      </c>
+      <c r="I7" s="67" t="n">
+        <v>290</v>
+      </c>
+      <c r="J7" s="67" t="n">
+        <v>350</v>
+      </c>
+      <c r="K7" s="67" t="n">
+        <v>382</v>
+      </c>
+      <c r="L7" s="67" t="n">
+        <v>484</v>
+      </c>
+      <c r="M7" s="67" t="n">
+        <v>505</v>
+      </c>
+      <c r="N7" s="67" t="n">
+        <v>441</v>
+      </c>
+      <c r="O7" s="67" t="n">
+        <v>415</v>
+      </c>
+      <c r="P7" s="67" t="n">
+        <v>485</v>
+      </c>
+      <c r="Q7" s="67" t="n">
+        <v>1457</v>
+      </c>
+      <c r="R7" s="67" t="n">
+        <v>1462</v>
+      </c>
+      <c r="S7" s="67" t="n">
+        <v>1454</v>
+      </c>
+      <c r="T7" s="67" t="n">
+        <v>1818</v>
+      </c>
+      <c r="U7" s="67" t="n">
+        <v>1892</v>
+      </c>
+      <c r="V7" s="67" t="n">
+        <v>1843</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="68" t="inlineStr">
+        <is>
+          <t>Managing Partner / CIO</t>
+        </is>
+      </c>
+      <c r="B8" s="69" t="n">
+        <v>0.4058853373921867</v>
+      </c>
+      <c r="C8" s="69" t="n">
+        <v>0.4181102358089466</v>
+      </c>
+      <c r="D8" s="69" t="n">
+        <v>0.4716981132075472</v>
+      </c>
+      <c r="E8" s="69" t="n">
+        <v>0.4086636480581222</v>
+      </c>
+      <c r="F8" s="69" t="n">
+        <v>0.3710155007741043</v>
+      </c>
+      <c r="G8" s="69" t="n">
+        <v>0.3740693678369545</v>
+      </c>
+      <c r="H8" s="69" t="n">
+        <v>0.3665146064743118</v>
+      </c>
+      <c r="I8" s="69" t="n">
+        <v>0.3160774852233587</v>
+      </c>
+      <c r="J8" s="69" t="n">
+        <v>0.2834731739911558</v>
+      </c>
+      <c r="K8" s="69" t="n">
+        <v>0.2681422535657876</v>
+      </c>
+      <c r="L8" s="69" t="n">
+        <v>0.2293236143202949</v>
+      </c>
+      <c r="M8" s="69" t="n">
+        <v>0.2237103228438481</v>
+      </c>
+      <c r="N8" s="69" t="n">
+        <v>0.2442902861034774</v>
+      </c>
+      <c r="O8" s="69" t="n">
+        <v>0.2543483353706967</v>
+      </c>
+      <c r="P8" s="69" t="n">
+        <v>0.2289710921190028</v>
+      </c>
+      <c r="Q8" s="69" t="n">
+        <v>0.1639623987109049</v>
+      </c>
+      <c r="R8" s="69" t="n">
+        <v>0.1637801712085247</v>
+      </c>
+      <c r="S8" s="69" t="n">
+        <v>0.1641121949179748</v>
+      </c>
+      <c r="T8" s="69" t="n">
+        <v>0.1502131462366411</v>
+      </c>
+      <c r="U8" s="69" t="n">
+        <v>0.1476627549294869</v>
+      </c>
+      <c r="V8" s="69" t="n">
+        <v>0.1493314823247189</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="70" t="inlineStr">
+        <is>
+          <t>Partner / Co-PM</t>
+        </is>
+      </c>
+      <c r="B9" s="71" t="n">
+        <v>0.243531202435312</v>
+      </c>
+      <c r="C9" s="71" t="n">
+        <v>0.250866141485368</v>
+      </c>
+      <c r="D9" s="71" t="n">
+        <v>0.2830188679245283</v>
+      </c>
+      <c r="E9" s="71" t="n">
+        <v>0.2451981888348733</v>
+      </c>
+      <c r="F9" s="71" t="n">
+        <v>0.2226093004644626</v>
+      </c>
+      <c r="G9" s="71" t="n">
+        <v>0.2244416207021727</v>
+      </c>
+      <c r="H9" s="71" t="n">
+        <v>0.2199087638845871</v>
+      </c>
+      <c r="I9" s="71" t="n">
+        <v>0.1896464911340152</v>
+      </c>
+      <c r="J9" s="71" t="n">
+        <v>0.2122853784665377</v>
+      </c>
+      <c r="K9" s="71" t="n">
+        <v>0.2269733893256809</v>
+      </c>
+      <c r="L9" s="71" t="n">
+        <v>0.2641641501512013</v>
+      </c>
+      <c r="M9" s="71" t="n">
+        <v>0.2684523874126177</v>
+      </c>
+      <c r="N9" s="71" t="n">
+        <v>0.2498251129911846</v>
+      </c>
+      <c r="O9" s="71" t="n">
+        <v>0.2401888528867841</v>
+      </c>
+      <c r="P9" s="71" t="n">
+        <v>0.2645018891634069</v>
+      </c>
+      <c r="Q9" s="71" t="n">
+        <v>0.241752041400785</v>
+      </c>
+      <c r="R9" s="71" t="n">
+        <v>0.2419135772641852</v>
+      </c>
+      <c r="S9" s="71" t="n">
+        <v>0.241619254311421</v>
+      </c>
+      <c r="T9" s="71" t="n">
+        <v>0.2539400884328099</v>
+      </c>
+      <c r="U9" s="71" t="n">
+        <v>0.256200886920571</v>
+      </c>
+      <c r="V9" s="71" t="n">
+        <v>0.2547216408295717</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="68" t="inlineStr">
+        <is>
+          <t>Portfolio Manager</t>
+        </is>
+      </c>
+      <c r="B10" s="69" t="n">
+        <v>0.05073566717402334</v>
+      </c>
+      <c r="C10" s="69" t="n">
+        <v>0.04131138184910298</v>
+      </c>
+      <c r="D10" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="69" t="n">
+        <v>0.04859384222428394</v>
+      </c>
+      <c r="F10" s="69" t="n">
+        <v>0.07761714122141777</v>
+      </c>
+      <c r="G10" s="69" t="n">
+        <v>0.07526288734023868</v>
+      </c>
+      <c r="H10" s="69" t="n">
+        <v>0.08108692155434877</v>
+      </c>
+      <c r="I10" s="69" t="n">
+        <v>0.1199693568459926</v>
+      </c>
+      <c r="J10" s="69" t="n">
+        <v>0.1133892695964623</v>
+      </c>
+      <c r="K10" s="69" t="n">
+        <v>0.107256901426315</v>
+      </c>
+      <c r="L10" s="69" t="n">
+        <v>0.09172944572811798</v>
+      </c>
+      <c r="M10" s="69" t="n">
+        <v>0.09045271413385651</v>
+      </c>
+      <c r="N10" s="69" t="n">
+        <v>0.09771611444139094</v>
+      </c>
+      <c r="O10" s="69" t="n">
+        <v>0.1017393341482787</v>
+      </c>
+      <c r="P10" s="69" t="n">
+        <v>0.09158843684760112</v>
+      </c>
+      <c r="Q10" s="69" t="n">
+        <v>0.1611680276005233</v>
+      </c>
+      <c r="R10" s="69" t="n">
+        <v>0.1612757181761235</v>
+      </c>
+      <c r="S10" s="69" t="n">
+        <v>0.1610795028742807</v>
+      </c>
+      <c r="T10" s="69" t="n">
+        <v>0.1692933922885399</v>
+      </c>
+      <c r="U10" s="69" t="n">
+        <v>0.1708005912803806</v>
+      </c>
+      <c r="V10" s="69" t="n">
+        <v>0.1698144272197145</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="70" t="inlineStr">
+        <is>
+          <t>Head of Research</t>
+        </is>
+      </c>
+      <c r="B11" s="71" t="n">
+        <v>0.0380517503805175</v>
+      </c>
+      <c r="C11" s="71" t="n">
+        <v>0.03098353638682724</v>
+      </c>
+      <c r="D11" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="71" t="n">
+        <v>0.03644538166821296</v>
+      </c>
+      <c r="F11" s="71" t="n">
+        <v>0.05821285591606334</v>
+      </c>
+      <c r="G11" s="71" t="n">
+        <v>0.05644716550517902</v>
+      </c>
+      <c r="H11" s="71" t="n">
+        <v>0.06081519116576158</v>
+      </c>
+      <c r="I11" s="71" t="n">
+        <v>0.08997701763449445</v>
+      </c>
+      <c r="J11" s="71" t="n">
+        <v>0.08504195219734675</v>
+      </c>
+      <c r="K11" s="71" t="n">
+        <v>0.08044267606973626</v>
+      </c>
+      <c r="L11" s="71" t="n">
+        <v>0.06879708429608848</v>
+      </c>
+      <c r="M11" s="71" t="n">
+        <v>0.06711309685315443</v>
+      </c>
+      <c r="N11" s="71" t="n">
+        <v>0.07328708583104321</v>
+      </c>
+      <c r="O11" s="71" t="n">
+        <v>0.07630450061120903</v>
+      </c>
+      <c r="P11" s="71" t="n">
+        <v>0.06869132763570084</v>
+      </c>
+      <c r="Q11" s="71" t="n">
+        <v>0.04918871961327147</v>
+      </c>
+      <c r="R11" s="71" t="n">
+        <v>0.04913405136255741</v>
+      </c>
+      <c r="S11" s="71" t="n">
+        <v>0.04923365847539245</v>
+      </c>
+      <c r="T11" s="71" t="n">
+        <v>0.04506394387099233</v>
+      </c>
+      <c r="U11" s="71" t="n">
+        <v>0.04429882647884606</v>
+      </c>
+      <c r="V11" s="71" t="n">
+        <v>0.04479944469741567</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="68" t="inlineStr">
+        <is>
+          <t>Senior Analyst</t>
+        </is>
+      </c>
+      <c r="B12" s="69" t="n">
+        <v>0.08117706747843734</v>
+      </c>
+      <c r="C12" s="69" t="n">
+        <v>0.08362204716178932</v>
+      </c>
+      <c r="D12" s="69" t="n">
+        <v>0.09433962264150944</v>
+      </c>
+      <c r="E12" s="69" t="n">
+        <v>0.08173272961162445</v>
+      </c>
+      <c r="F12" s="69" t="n">
+        <v>0.07420310015482087</v>
+      </c>
+      <c r="G12" s="69" t="n">
+        <v>0.07481387356739091</v>
+      </c>
+      <c r="H12" s="69" t="n">
+        <v>0.07330292129486236</v>
+      </c>
+      <c r="I12" s="69" t="n">
+        <v>0.06321549704467173</v>
+      </c>
+      <c r="J12" s="69" t="n">
+        <v>0.07076179282217923</v>
+      </c>
+      <c r="K12" s="69" t="n">
+        <v>0.07565779644189363</v>
+      </c>
+      <c r="L12" s="69" t="n">
+        <v>0.08805471671706708</v>
+      </c>
+      <c r="M12" s="69" t="n">
+        <v>0.08996842163569788</v>
+      </c>
+      <c r="N12" s="69" t="n">
+        <v>0.08327503766372819</v>
+      </c>
+      <c r="O12" s="69" t="n">
+        <v>0.08006295096226136</v>
+      </c>
+      <c r="P12" s="69" t="n">
+        <v>0.08816729638780231</v>
+      </c>
+      <c r="Q12" s="69" t="n">
+        <v>0.1133764935424426</v>
+      </c>
+      <c r="R12" s="69" t="n">
+        <v>0.1133938933297667</v>
+      </c>
+      <c r="S12" s="69" t="n">
+        <v>0.1133621904207353</v>
+      </c>
+      <c r="T12" s="69" t="n">
+        <v>0.1146893253915982</v>
+      </c>
+      <c r="U12" s="69" t="n">
+        <v>0.1149328466260877</v>
+      </c>
+      <c r="V12" s="69" t="n">
+        <v>0.114773510074801</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="70" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="B13" s="71" t="n">
+        <v>0.0639269406392694</v>
+      </c>
+      <c r="C13" s="71" t="n">
+        <v>0.06256664285180449</v>
+      </c>
+      <c r="D13" s="71" t="n">
+        <v>0.05660377358490566</v>
+      </c>
+      <c r="E13" s="71" t="n">
+        <v>0.06361779043425984</v>
+      </c>
+      <c r="F13" s="71" t="n">
+        <v>0.06780700245931787</v>
+      </c>
+      <c r="G13" s="71" t="n">
+        <v>0.06746719034250616</v>
+      </c>
+      <c r="H13" s="71" t="n">
+        <v>0.06830782924322205</v>
+      </c>
+      <c r="I13" s="71" t="n">
+        <v>0.07392010528060082</v>
+      </c>
+      <c r="J13" s="71" t="n">
+        <v>0.07647385657224623</v>
+      </c>
+      <c r="K13" s="71" t="n">
+        <v>0.07757174829303069</v>
+      </c>
+      <c r="L13" s="71" t="n">
+        <v>0.08035166374867565</v>
+      </c>
+      <c r="M13" s="71" t="n">
+        <v>0.08082629172268051</v>
+      </c>
+      <c r="N13" s="71" t="n">
+        <v>0.0792798569306542</v>
+      </c>
+      <c r="O13" s="71" t="n">
+        <v>0.07855957082184042</v>
+      </c>
+      <c r="P13" s="71" t="n">
+        <v>0.08037690888696172</v>
+      </c>
+      <c r="Q13" s="71" t="n">
+        <v>0.096700816560314</v>
+      </c>
+      <c r="R13" s="71" t="n">
+        <v>0.09676543090567409</v>
+      </c>
+      <c r="S13" s="71" t="n">
+        <v>0.09664770172456839</v>
+      </c>
+      <c r="T13" s="71" t="n">
+        <v>0.1015760353731239</v>
+      </c>
+      <c r="U13" s="71" t="n">
+        <v>0.1024803547682284</v>
+      </c>
+      <c r="V13" s="71" t="n">
+        <v>0.1018886563318287</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="68" t="inlineStr">
+        <is>
+          <t>Junior Analyst</t>
+        </is>
+      </c>
+      <c r="B14" s="69" t="n">
+        <v>0.0076103500761035</v>
+      </c>
+      <c r="C14" s="69" t="n">
+        <v>0.006196707277365446</v>
+      </c>
+      <c r="D14" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="69" t="n">
+        <v>0.007289076333642593</v>
+      </c>
+      <c r="F14" s="69" t="n">
+        <v>0.01164257118321267</v>
+      </c>
+      <c r="G14" s="69" t="n">
+        <v>0.0112894331010358</v>
+      </c>
+      <c r="H14" s="69" t="n">
+        <v>0.01216303823315231</v>
+      </c>
+      <c r="I14" s="69" t="n">
+        <v>0.01799540352689889</v>
+      </c>
+      <c r="J14" s="69" t="n">
+        <v>0.02122853784665377</v>
+      </c>
+      <c r="K14" s="69" t="n">
+        <v>0.02269733893256809</v>
+      </c>
+      <c r="L14" s="69" t="n">
+        <v>0.02641641501512013</v>
+      </c>
+      <c r="M14" s="69" t="n">
+        <v>0.02699052649070936</v>
+      </c>
+      <c r="N14" s="69" t="n">
+        <v>0.02498251129911846</v>
+      </c>
+      <c r="O14" s="69" t="n">
+        <v>0.02401888528867841</v>
+      </c>
+      <c r="P14" s="69" t="n">
+        <v>0.02645018891634069</v>
+      </c>
+      <c r="Q14" s="69" t="n">
+        <v>0.03401294806273279</v>
+      </c>
+      <c r="R14" s="69" t="n">
+        <v>0.03401816799893</v>
+      </c>
+      <c r="S14" s="69" t="n">
+        <v>0.03400865712622059</v>
+      </c>
+      <c r="T14" s="69" t="n">
+        <v>0.03440679761747945</v>
+      </c>
+      <c r="U14" s="69" t="n">
+        <v>0.03447985398782631</v>
+      </c>
+      <c r="V14" s="69" t="n">
+        <v>0.0344320530224403</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="70" t="inlineStr">
+        <is>
+          <t>Head of Trading</t>
+        </is>
+      </c>
+      <c r="B15" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="71" t="n">
+        <v>0.01266044222155325</v>
+      </c>
+      <c r="K15" s="71" t="n">
+        <v>0.01982641115586252</v>
+      </c>
+      <c r="L15" s="71" t="n">
+        <v>0.03797099446770729</v>
+      </c>
+      <c r="M15" s="71" t="n">
+        <v>0.04026785811189266</v>
+      </c>
+      <c r="N15" s="71" t="n">
+        <v>0.03097528239872945</v>
+      </c>
+      <c r="O15" s="71" t="n">
+        <v>0.02627395549930982</v>
+      </c>
+      <c r="P15" s="71" t="n">
+        <v>0.03813577016760158</v>
+      </c>
+      <c r="Q15" s="71" t="n">
+        <v>0.02951323176796288</v>
+      </c>
+      <c r="R15" s="71" t="n">
+        <v>0.02948043081753444</v>
+      </c>
+      <c r="S15" s="71" t="n">
+        <v>0.02954019508523547</v>
+      </c>
+      <c r="T15" s="71" t="n">
+        <v>0.0270383663225954</v>
+      </c>
+      <c r="U15" s="71" t="n">
+        <v>0.02657929588730763</v>
+      </c>
+      <c r="V15" s="71" t="n">
+        <v>0.02687966681844941</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="68" t="inlineStr">
+        <is>
+          <t>Trader / Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="69" t="n">
+        <v>0.01268391679350583</v>
+      </c>
+      <c r="C16" s="69" t="n">
+        <v>0.01032784546227574</v>
+      </c>
+      <c r="D16" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="69" t="n">
+        <v>0.01214846055607099</v>
+      </c>
+      <c r="F16" s="69" t="n">
+        <v>0.01940428530535444</v>
+      </c>
+      <c r="G16" s="69" t="n">
+        <v>0.01881572183505967</v>
+      </c>
+      <c r="H16" s="69" t="n">
+        <v>0.02027173038858719</v>
+      </c>
+      <c r="I16" s="69" t="n">
+        <v>0.02999233921149815</v>
+      </c>
+      <c r="J16" s="69" t="n">
+        <v>0.02834731739911558</v>
+      </c>
+      <c r="K16" s="69" t="n">
+        <v>0.02681422535657876</v>
+      </c>
+      <c r="L16" s="69" t="n">
+        <v>0.02293236143202949</v>
+      </c>
+      <c r="M16" s="69" t="n">
+        <v>0.02261317853346413</v>
+      </c>
+      <c r="N16" s="69" t="n">
+        <v>0.02442902861034774</v>
+      </c>
+      <c r="O16" s="69" t="n">
+        <v>0.02543483353706967</v>
+      </c>
+      <c r="P16" s="69" t="n">
+        <v>0.02289710921190028</v>
+      </c>
+      <c r="Q16" s="69" t="n">
+        <v>0.03279247974218098</v>
+      </c>
+      <c r="R16" s="69" t="n">
+        <v>0.03275603424170494</v>
+      </c>
+      <c r="S16" s="69" t="n">
+        <v>0.03282243898359496</v>
+      </c>
+      <c r="T16" s="69" t="n">
+        <v>0.03004262924732822</v>
+      </c>
+      <c r="U16" s="69" t="n">
+        <v>0.02953255098589737</v>
+      </c>
+      <c r="V16" s="69" t="n">
+        <v>0.02986629646494378</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="70" t="inlineStr">
+        <is>
+          <t>COO / Head of Operations</t>
+        </is>
+      </c>
+      <c r="B17" s="71" t="n">
+        <v>0.060882800608828</v>
+      </c>
+      <c r="C17" s="71" t="n">
+        <v>0.062716535371342</v>
+      </c>
+      <c r="D17" s="71" t="n">
+        <v>0.07075471698113207</v>
+      </c>
+      <c r="E17" s="71" t="n">
+        <v>0.06129954720871834</v>
+      </c>
+      <c r="F17" s="71" t="n">
+        <v>0.05565232511611565</v>
+      </c>
+      <c r="G17" s="71" t="n">
+        <v>0.05611040517554319</v>
+      </c>
+      <c r="H17" s="71" t="n">
+        <v>0.05497719097114678</v>
+      </c>
+      <c r="I17" s="71" t="n">
+        <v>0.0474116227835038</v>
+      </c>
+      <c r="J17" s="71" t="n">
+        <v>0.04252097609867338</v>
+      </c>
+      <c r="K17" s="71" t="n">
+        <v>0.04022133803486813</v>
+      </c>
+      <c r="L17" s="71" t="n">
+        <v>0.03439854214804424</v>
+      </c>
+      <c r="M17" s="71" t="n">
+        <v>0.03355654842657722</v>
+      </c>
+      <c r="N17" s="71" t="n">
+        <v>0.0366435429155216</v>
+      </c>
+      <c r="O17" s="71" t="n">
+        <v>0.03815225030560451</v>
+      </c>
+      <c r="P17" s="71" t="n">
+        <v>0.03434566381785042</v>
+      </c>
+      <c r="Q17" s="71" t="n">
+        <v>0.02459435980663573</v>
+      </c>
+      <c r="R17" s="71" t="n">
+        <v>0.0245670256812787</v>
+      </c>
+      <c r="S17" s="71" t="n">
+        <v>0.02461682923769622</v>
+      </c>
+      <c r="T17" s="71" t="n">
+        <v>0.02253197193549616</v>
+      </c>
+      <c r="U17" s="71" t="n">
+        <v>0.02214941323942303</v>
+      </c>
+      <c r="V17" s="71" t="n">
+        <v>0.02239972234870784</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="68" t="inlineStr">
+        <is>
+          <t>CFO / Finance</t>
+        </is>
+      </c>
+      <c r="B18" s="69" t="n">
+        <v>0.015220700152207</v>
+      </c>
+      <c r="C18" s="69" t="n">
+        <v>0.01239341455473089</v>
+      </c>
+      <c r="D18" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="69" t="n">
+        <v>0.01457815266728519</v>
+      </c>
+      <c r="F18" s="69" t="n">
+        <v>0.02328514236642533</v>
+      </c>
+      <c r="G18" s="69" t="n">
+        <v>0.02257886620207161</v>
+      </c>
+      <c r="H18" s="69" t="n">
+        <v>0.02432607646630463</v>
+      </c>
+      <c r="I18" s="69" t="n">
+        <v>0.03599080705379777</v>
+      </c>
+      <c r="J18" s="69" t="n">
+        <v>0.0340167808789387</v>
+      </c>
+      <c r="K18" s="69" t="n">
+        <v>0.03217707042789451</v>
+      </c>
+      <c r="L18" s="69" t="n">
+        <v>0.02751883371843539</v>
+      </c>
+      <c r="M18" s="69" t="n">
+        <v>0.02684523874126177</v>
+      </c>
+      <c r="N18" s="69" t="n">
+        <v>0.02931483433241728</v>
+      </c>
+      <c r="O18" s="69" t="n">
+        <v>0.03052180024448361</v>
+      </c>
+      <c r="P18" s="69" t="n">
+        <v>0.02747653105428034</v>
+      </c>
+      <c r="Q18" s="69" t="n">
+        <v>0.01967548784530859</v>
+      </c>
+      <c r="R18" s="69" t="n">
+        <v>0.01965362054502296</v>
+      </c>
+      <c r="S18" s="69" t="n">
+        <v>0.01969346339015698</v>
+      </c>
+      <c r="T18" s="69" t="n">
+        <v>0.01802557754839693</v>
+      </c>
+      <c r="U18" s="69" t="n">
+        <v>0.01771953059153842</v>
+      </c>
+      <c r="V18" s="69" t="n">
+        <v>0.01791977787896627</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="70" t="inlineStr">
+        <is>
+          <t>Compliance / Legal</t>
+        </is>
+      </c>
+      <c r="B19" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="71" t="n">
+        <v>0.00562686320957922</v>
+      </c>
+      <c r="K19" s="71" t="n">
+        <v>0.008811738291494453</v>
+      </c>
+      <c r="L19" s="71" t="n">
+        <v>0.01687599754120324</v>
+      </c>
+      <c r="M19" s="71" t="n">
+        <v>0.01789682582750785</v>
+      </c>
+      <c r="N19" s="71" t="n">
+        <v>0.01376679217721309</v>
+      </c>
+      <c r="O19" s="71" t="n">
+        <v>0.01167731355524881</v>
+      </c>
+      <c r="P19" s="71" t="n">
+        <v>0.0169492311856007</v>
+      </c>
+      <c r="Q19" s="71" t="n">
+        <v>0.01311699189687239</v>
+      </c>
+      <c r="R19" s="71" t="n">
+        <v>0.01310241369668197</v>
+      </c>
+      <c r="S19" s="71" t="n">
+        <v>0.01312897559343799</v>
+      </c>
+      <c r="T19" s="71" t="n">
+        <v>0.01201705169893129</v>
+      </c>
+      <c r="U19" s="71" t="n">
+        <v>0.01181302039435895</v>
+      </c>
+      <c r="V19" s="71" t="n">
+        <v>0.01194651858597751</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="68" t="inlineStr">
+        <is>
+          <t>Investor Relations / Ops</t>
+        </is>
+      </c>
+      <c r="B20" s="69" t="n">
+        <v>0.02029426686960933</v>
+      </c>
+      <c r="C20" s="69" t="n">
+        <v>0.02090551179044733</v>
+      </c>
+      <c r="D20" s="69" t="n">
+        <v>0.02358490566037736</v>
+      </c>
+      <c r="E20" s="69" t="n">
+        <v>0.02043318240290611</v>
+      </c>
+      <c r="F20" s="69" t="n">
+        <v>0.01855077503870522</v>
+      </c>
+      <c r="G20" s="69" t="n">
+        <v>0.01870346839184773</v>
+      </c>
+      <c r="H20" s="69" t="n">
+        <v>0.01832573032371559</v>
+      </c>
+      <c r="I20" s="69" t="n">
+        <v>0.01580387426116793</v>
+      </c>
+      <c r="J20" s="69" t="n">
+        <v>0.01417365869955779</v>
+      </c>
+      <c r="K20" s="69" t="n">
+        <v>0.01340711267828938</v>
+      </c>
+      <c r="L20" s="69" t="n">
+        <v>0.01146618071601475</v>
+      </c>
+      <c r="M20" s="69" t="n">
+        <v>0.01130658926673206</v>
+      </c>
+      <c r="N20" s="69" t="n">
+        <v>0.01221451430517387</v>
+      </c>
+      <c r="O20" s="69" t="n">
+        <v>0.01271741676853484</v>
+      </c>
+      <c r="P20" s="69" t="n">
+        <v>0.01144855460595014</v>
+      </c>
+      <c r="Q20" s="69" t="n">
+        <v>0.02014600345006541</v>
+      </c>
+      <c r="R20" s="69" t="n">
+        <v>0.02015946477201543</v>
+      </c>
+      <c r="S20" s="69" t="n">
+        <v>0.02013493785928508</v>
+      </c>
+      <c r="T20" s="69" t="n">
+        <v>0.02116167403606749</v>
+      </c>
+      <c r="U20" s="69" t="n">
+        <v>0.02135007391004758</v>
+      </c>
+      <c r="V20" s="69" t="n">
+        <v>0.02122680340246431</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="72" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B21" s="73">
+        <f>SUM(B8:B20)</f>
+        <v/>
+      </c>
+      <c r="C21" s="73">
+        <f>SUM(C8:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="73">
+        <f>SUM(D8:D20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="73">
+        <f>SUM(E8:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="73">
+        <f>SUM(F8:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="73">
+        <f>SUM(G8:G20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="73">
+        <f>SUM(H8:H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="73">
+        <f>SUM(I8:I20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="73">
+        <f>SUM(J8:J20)</f>
+        <v/>
+      </c>
+      <c r="K21" s="73">
+        <f>SUM(K8:K20)</f>
+        <v/>
+      </c>
+      <c r="L21" s="73">
+        <f>SUM(L8:L20)</f>
+        <v/>
+      </c>
+      <c r="M21" s="73">
+        <f>SUM(M8:M20)</f>
+        <v/>
+      </c>
+      <c r="N21" s="73">
+        <f>SUM(N8:N20)</f>
+        <v/>
+      </c>
+      <c r="O21" s="73">
+        <f>SUM(O8:O20)</f>
+        <v/>
+      </c>
+      <c r="P21" s="73">
+        <f>SUM(P8:P20)</f>
+        <v/>
+      </c>
+      <c r="Q21" s="73">
+        <f>SUM(Q8:Q20)</f>
+        <v/>
+      </c>
+      <c r="R21" s="73">
+        <f>SUM(R8:R20)</f>
+        <v/>
+      </c>
+      <c r="S21" s="73">
+        <f>SUM(S8:S20)</f>
+        <v/>
+      </c>
+      <c r="T21" s="73">
+        <f>SUM(T8:T20)</f>
+        <v/>
+      </c>
+      <c r="U21" s="73">
+        <f>SUM(U8:U20)</f>
+        <v/>
+      </c>
+      <c r="V21" s="73">
+        <f>SUM(V8:V20)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:V2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A1:V1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Replace time-based take analysis with AUM sweep $100m -> $2bn
Drops the historical-return AUM path. New 'Take by AUM' sheet sweeps AUM
smoothly from $100m to $2bn (20 steps), interpolating headcount across the
scenarios and computing each role's % of the take at each AUM level. Adds a
native Excel line chart and a stacked-area PNG.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K14qB8MpeJ8Pk8H1GeEUV4
</commit_message>
<xml_diff>
--- a/Performance_Fee_Framework.xlsx
+++ b/Performance_Fee_Framework.xlsx
@@ -7,7 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Static" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Take Over Time" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Take by AUM" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Sheet1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -330,7 +330,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -491,6 +491,9 @@
     <xf numFmtId="9" fontId="25" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="25" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -581,7 +584,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Role share of the take over time (%)</a:t>
+              <a:t>Role share of the take vs AUM</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -595,7 +598,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A8</f>
+              <f>'Take by AUM'!A5</f>
             </strRef>
           </tx>
           <spPr>
@@ -613,12 +616,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$8:$V$8</f>
+              <f>'Take by AUM'!$B$5:$U$5</f>
             </numRef>
           </val>
         </ser>
@@ -627,7 +630,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A9</f>
+              <f>'Take by AUM'!A6</f>
             </strRef>
           </tx>
           <spPr>
@@ -645,12 +648,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$9:$V$9</f>
+              <f>'Take by AUM'!$B$6:$U$6</f>
             </numRef>
           </val>
         </ser>
@@ -659,7 +662,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A10</f>
+              <f>'Take by AUM'!A7</f>
             </strRef>
           </tx>
           <spPr>
@@ -677,12 +680,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$10:$V$10</f>
+              <f>'Take by AUM'!$B$7:$U$7</f>
             </numRef>
           </val>
         </ser>
@@ -691,7 +694,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A11</f>
+              <f>'Take by AUM'!A8</f>
             </strRef>
           </tx>
           <spPr>
@@ -709,12 +712,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$11:$V$11</f>
+              <f>'Take by AUM'!$B$8:$U$8</f>
             </numRef>
           </val>
         </ser>
@@ -723,7 +726,7 @@
           <order val="4"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A12</f>
+              <f>'Take by AUM'!A9</f>
             </strRef>
           </tx>
           <spPr>
@@ -741,12 +744,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$12:$V$12</f>
+              <f>'Take by AUM'!$B$9:$U$9</f>
             </numRef>
           </val>
         </ser>
@@ -755,7 +758,7 @@
           <order val="5"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A13</f>
+              <f>'Take by AUM'!A10</f>
             </strRef>
           </tx>
           <spPr>
@@ -773,12 +776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$13:$V$13</f>
+              <f>'Take by AUM'!$B$10:$U$10</f>
             </numRef>
           </val>
         </ser>
@@ -787,7 +790,7 @@
           <order val="6"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A14</f>
+              <f>'Take by AUM'!A11</f>
             </strRef>
           </tx>
           <spPr>
@@ -805,12 +808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$14:$V$14</f>
+              <f>'Take by AUM'!$B$11:$U$11</f>
             </numRef>
           </val>
         </ser>
@@ -819,7 +822,7 @@
           <order val="7"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A15</f>
+              <f>'Take by AUM'!A12</f>
             </strRef>
           </tx>
           <spPr>
@@ -837,12 +840,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$15:$V$15</f>
+              <f>'Take by AUM'!$B$12:$U$12</f>
             </numRef>
           </val>
         </ser>
@@ -851,7 +854,7 @@
           <order val="8"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A16</f>
+              <f>'Take by AUM'!A13</f>
             </strRef>
           </tx>
           <spPr>
@@ -869,12 +872,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$16:$V$16</f>
+              <f>'Take by AUM'!$B$13:$U$13</f>
             </numRef>
           </val>
         </ser>
@@ -883,7 +886,7 @@
           <order val="9"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A17</f>
+              <f>'Take by AUM'!A14</f>
             </strRef>
           </tx>
           <spPr>
@@ -901,12 +904,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$17:$V$17</f>
+              <f>'Take by AUM'!$B$14:$U$14</f>
             </numRef>
           </val>
         </ser>
@@ -915,7 +918,7 @@
           <order val="10"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A18</f>
+              <f>'Take by AUM'!A15</f>
             </strRef>
           </tx>
           <spPr>
@@ -933,12 +936,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$18:$V$18</f>
+              <f>'Take by AUM'!$B$15:$U$15</f>
             </numRef>
           </val>
         </ser>
@@ -947,7 +950,7 @@
           <order val="11"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A19</f>
+              <f>'Take by AUM'!A16</f>
             </strRef>
           </tx>
           <spPr>
@@ -965,12 +968,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$19:$V$19</f>
+              <f>'Take by AUM'!$B$16:$U$16</f>
             </numRef>
           </val>
         </ser>
@@ -979,7 +982,7 @@
           <order val="12"/>
           <tx>
             <strRef>
-              <f>'Take Over Time'!A20</f>
+              <f>'Take by AUM'!A17</f>
             </strRef>
           </tx>
           <spPr>
@@ -997,12 +1000,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Take Over Time'!$B$6:$V$6</f>
+              <f>'Take by AUM'!$B$4:$U$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Take Over Time'!$B$20:$V$20</f>
+              <f>'Take by AUM'!$B$17:$U$17</f>
             </numRef>
           </val>
         </ser>
@@ -1024,7 +1027,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Year</a:t>
+                  <a:t>AUM (USD m)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1104,7 +1107,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9360000" cy="3960000"/>
@@ -4026,7 +4029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4050,1179 +4053,1051 @@
     <col width="7" customWidth="1" min="19" max="19"/>
     <col width="7" customWidth="1" min="20" max="20"/>
     <col width="7" customWidth="1" min="21" max="21"/>
-    <col width="7" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="61" t="inlineStr">
         <is>
-          <t>Each role's share of the take (comp pool), over time</t>
+          <t>Each role's share of the take (comp pool) as AUM grows $100m → $2bn</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>Share = role weight × headcount ÷ total weighted units. Headcount scales with the AUM path; % sums to 100% each year.</t>
+          <t>Share = role weight × headcount ÷ total weighted units. Headcount interpolated across the AUM scenarios. Columns sum to 100%.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="63" t="inlineStr">
-        <is>
-          <t>Starting AUM (USD m), compounded by Athanase net returns:</t>
-        </is>
-      </c>
-      <c r="D4" s="64" t="n">
+      <c r="A4" s="72" t="inlineStr">
+        <is>
+          <t>AUM (USD m) →</t>
+        </is>
+      </c>
+      <c r="B4" s="74" t="n">
         <v>100</v>
       </c>
+      <c r="C4" s="74" t="n">
+        <v>200</v>
+      </c>
+      <c r="D4" s="74" t="n">
+        <v>300</v>
+      </c>
+      <c r="E4" s="74" t="n">
+        <v>400</v>
+      </c>
+      <c r="F4" s="74" t="n">
+        <v>500</v>
+      </c>
+      <c r="G4" s="74" t="n">
+        <v>600</v>
+      </c>
+      <c r="H4" s="74" t="n">
+        <v>700</v>
+      </c>
+      <c r="I4" s="74" t="n">
+        <v>800</v>
+      </c>
+      <c r="J4" s="74" t="n">
+        <v>900</v>
+      </c>
+      <c r="K4" s="74" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L4" s="74" t="n">
+        <v>1100</v>
+      </c>
+      <c r="M4" s="74" t="n">
+        <v>1200</v>
+      </c>
+      <c r="N4" s="74" t="n">
+        <v>1300</v>
+      </c>
+      <c r="O4" s="74" t="n">
+        <v>1400</v>
+      </c>
+      <c r="P4" s="74" t="n">
+        <v>1500</v>
+      </c>
+      <c r="Q4" s="74" t="n">
+        <v>1600</v>
+      </c>
+      <c r="R4" s="74" t="n">
+        <v>1700</v>
+      </c>
+      <c r="S4" s="74" t="n">
+        <v>1800</v>
+      </c>
+      <c r="T4" s="74" t="n">
+        <v>1900</v>
+      </c>
+      <c r="U4" s="74" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="68" t="inlineStr">
+        <is>
+          <t>Managing Partner / CIO</t>
+        </is>
+      </c>
+      <c r="B5" s="69" t="n">
+        <v>0.4716981132075472</v>
+      </c>
+      <c r="C5" s="69" t="n">
+        <v>0.3745318352059925</v>
+      </c>
+      <c r="D5" s="69" t="n">
+        <v>0.3105590062111801</v>
+      </c>
+      <c r="E5" s="69" t="n">
+        <v>0.2604166666666667</v>
+      </c>
+      <c r="F5" s="69" t="n">
+        <v>0.2242152466367713</v>
+      </c>
+      <c r="G5" s="69" t="n">
+        <v>0.2152389151958674</v>
+      </c>
+      <c r="H5" s="69" t="n">
+        <v>0.206953642384106</v>
+      </c>
+      <c r="I5" s="69" t="n">
+        <v>0.1992825827022718</v>
+      </c>
+      <c r="J5" s="69" t="n">
+        <v>0.1921598770176787</v>
+      </c>
+      <c r="K5" s="69" t="n">
+        <v>0.1855287569573284</v>
+      </c>
+      <c r="L5" s="69" t="n">
+        <v>0.1803426510369703</v>
+      </c>
+      <c r="M5" s="69" t="n">
+        <v>0.1754385964912281</v>
+      </c>
+      <c r="N5" s="69" t="n">
+        <v>0.1707941929974381</v>
+      </c>
+      <c r="O5" s="69" t="n">
+        <v>0.1663893510815308</v>
+      </c>
+      <c r="P5" s="69" t="n">
+        <v>0.16220600162206</v>
+      </c>
+      <c r="Q5" s="69" t="n">
+        <v>0.1582278481012658</v>
+      </c>
+      <c r="R5" s="69" t="n">
+        <v>0.1544401544401544</v>
+      </c>
+      <c r="S5" s="69" t="n">
+        <v>0.1508295625942685</v>
+      </c>
+      <c r="T5" s="69" t="n">
+        <v>0.1473839351510685</v>
+      </c>
+      <c r="U5" s="69" t="n">
+        <v>0.1440922190201729</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="65" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B6" s="65" t="n">
-        <v>2006</v>
-      </c>
-      <c r="C6" s="65" t="n">
-        <v>2007</v>
-      </c>
-      <c r="D6" s="65" t="n">
-        <v>2008</v>
-      </c>
-      <c r="E6" s="65" t="n">
-        <v>2009</v>
-      </c>
-      <c r="F6" s="65" t="n">
-        <v>2010</v>
-      </c>
-      <c r="G6" s="65" t="n">
-        <v>2011</v>
-      </c>
-      <c r="H6" s="65" t="n">
-        <v>2012</v>
-      </c>
-      <c r="I6" s="65" t="n">
-        <v>2013</v>
-      </c>
-      <c r="J6" s="65" t="n">
-        <v>2014</v>
-      </c>
-      <c r="K6" s="65" t="n">
-        <v>2015</v>
-      </c>
-      <c r="L6" s="65" t="n">
-        <v>2016</v>
-      </c>
-      <c r="M6" s="65" t="n">
-        <v>2017</v>
-      </c>
-      <c r="N6" s="65" t="n">
-        <v>2018</v>
-      </c>
-      <c r="O6" s="65" t="n">
-        <v>2019</v>
-      </c>
-      <c r="P6" s="65" t="n">
-        <v>2020</v>
-      </c>
-      <c r="Q6" s="65" t="n">
-        <v>2021</v>
-      </c>
-      <c r="R6" s="65" t="n">
-        <v>2022</v>
-      </c>
-      <c r="S6" s="65" t="n">
-        <v>2023</v>
-      </c>
-      <c r="T6" s="65" t="n">
-        <v>2024</v>
-      </c>
-      <c r="U6" s="65" t="n">
-        <v>2025</v>
-      </c>
-      <c r="V6" s="65" t="n">
-        <v>2026</v>
+      <c r="A6" s="70" t="inlineStr">
+        <is>
+          <t>Partner / Co-PM</t>
+        </is>
+      </c>
+      <c r="B6" s="71" t="n">
+        <v>0.2830188679245283</v>
+      </c>
+      <c r="C6" s="71" t="n">
+        <v>0.2247191011235955</v>
+      </c>
+      <c r="D6" s="71" t="n">
+        <v>0.1863354037267081</v>
+      </c>
+      <c r="E6" s="71" t="n">
+        <v>0.234375</v>
+      </c>
+      <c r="F6" s="71" t="n">
+        <v>0.2690582959641256</v>
+      </c>
+      <c r="G6" s="71" t="n">
+        <v>0.2582866982350409</v>
+      </c>
+      <c r="H6" s="71" t="n">
+        <v>0.2483443708609272</v>
+      </c>
+      <c r="I6" s="71" t="n">
+        <v>0.2391390992427262</v>
+      </c>
+      <c r="J6" s="71" t="n">
+        <v>0.2305918524212144</v>
+      </c>
+      <c r="K6" s="71" t="n">
+        <v>0.2226345083487941</v>
+      </c>
+      <c r="L6" s="71" t="n">
+        <v>0.2272317403065825</v>
+      </c>
+      <c r="M6" s="71" t="n">
+        <v>0.2315789473684211</v>
+      </c>
+      <c r="N6" s="71" t="n">
+        <v>0.2356959863364645</v>
+      </c>
+      <c r="O6" s="71" t="n">
+        <v>0.2396006655574043</v>
+      </c>
+      <c r="P6" s="71" t="n">
+        <v>0.24330900243309</v>
+      </c>
+      <c r="Q6" s="71" t="n">
+        <v>0.2468354430379747</v>
+      </c>
+      <c r="R6" s="71" t="n">
+        <v>0.2501930501930502</v>
+      </c>
+      <c r="S6" s="71" t="n">
+        <v>0.253393665158371</v>
+      </c>
+      <c r="T6" s="71" t="n">
+        <v>0.2564480471628592</v>
+      </c>
+      <c r="U6" s="71" t="n">
+        <v>0.2593659942363112</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="66" t="inlineStr">
-        <is>
-          <t>AUM (USD m)</t>
-        </is>
-      </c>
-      <c r="B7" s="67" t="n">
-        <v>162</v>
-      </c>
-      <c r="C7" s="67" t="n">
-        <v>149</v>
-      </c>
-      <c r="D7" s="67" t="n">
-        <v>88</v>
-      </c>
-      <c r="E7" s="67" t="n">
-        <v>159</v>
-      </c>
-      <c r="F7" s="67" t="n">
-        <v>205</v>
-      </c>
-      <c r="G7" s="67" t="n">
-        <v>201</v>
-      </c>
-      <c r="H7" s="67" t="n">
-        <v>211</v>
-      </c>
-      <c r="I7" s="67" t="n">
-        <v>290</v>
-      </c>
-      <c r="J7" s="67" t="n">
-        <v>350</v>
-      </c>
-      <c r="K7" s="67" t="n">
-        <v>382</v>
-      </c>
-      <c r="L7" s="67" t="n">
-        <v>484</v>
-      </c>
-      <c r="M7" s="67" t="n">
-        <v>505</v>
-      </c>
-      <c r="N7" s="67" t="n">
-        <v>441</v>
-      </c>
-      <c r="O7" s="67" t="n">
-        <v>415</v>
-      </c>
-      <c r="P7" s="67" t="n">
-        <v>485</v>
-      </c>
-      <c r="Q7" s="67" t="n">
-        <v>1457</v>
-      </c>
-      <c r="R7" s="67" t="n">
-        <v>1462</v>
-      </c>
-      <c r="S7" s="67" t="n">
-        <v>1454</v>
-      </c>
-      <c r="T7" s="67" t="n">
-        <v>1818</v>
-      </c>
-      <c r="U7" s="67" t="n">
-        <v>1892</v>
-      </c>
-      <c r="V7" s="67" t="n">
-        <v>1843</v>
+      <c r="A7" s="68" t="inlineStr">
+        <is>
+          <t>Portfolio Manager</t>
+        </is>
+      </c>
+      <c r="B7" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="69" t="n">
+        <v>0.0749063670411985</v>
+      </c>
+      <c r="D7" s="69" t="n">
+        <v>0.124223602484472</v>
+      </c>
+      <c r="E7" s="69" t="n">
+        <v>0.1041666666666667</v>
+      </c>
+      <c r="F7" s="69" t="n">
+        <v>0.08968609865470852</v>
+      </c>
+      <c r="G7" s="69" t="n">
+        <v>0.1033146792940164</v>
+      </c>
+      <c r="H7" s="69" t="n">
+        <v>0.1158940397350993</v>
+      </c>
+      <c r="I7" s="69" t="n">
+        <v>0.127540852929454</v>
+      </c>
+      <c r="J7" s="69" t="n">
+        <v>0.1383551114527286</v>
+      </c>
+      <c r="K7" s="69" t="n">
+        <v>0.1484230055658627</v>
+      </c>
+      <c r="L7" s="69" t="n">
+        <v>0.151487826871055</v>
+      </c>
+      <c r="M7" s="69" t="n">
+        <v>0.1543859649122807</v>
+      </c>
+      <c r="N7" s="69" t="n">
+        <v>0.157130657557643</v>
+      </c>
+      <c r="O7" s="69" t="n">
+        <v>0.1597337770382695</v>
+      </c>
+      <c r="P7" s="69" t="n">
+        <v>0.16220600162206</v>
+      </c>
+      <c r="Q7" s="69" t="n">
+        <v>0.1645569620253164</v>
+      </c>
+      <c r="R7" s="69" t="n">
+        <v>0.1667953667953668</v>
+      </c>
+      <c r="S7" s="69" t="n">
+        <v>0.1689291101055807</v>
+      </c>
+      <c r="T7" s="69" t="n">
+        <v>0.1709653647752395</v>
+      </c>
+      <c r="U7" s="69" t="n">
+        <v>0.1729106628242075</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="68" t="inlineStr">
-        <is>
-          <t>Managing Partner / CIO</t>
-        </is>
-      </c>
-      <c r="B8" s="69" t="n">
-        <v>0.4058853373921867</v>
-      </c>
-      <c r="C8" s="69" t="n">
-        <v>0.4181102358089466</v>
-      </c>
-      <c r="D8" s="69" t="n">
-        <v>0.4716981132075472</v>
-      </c>
-      <c r="E8" s="69" t="n">
-        <v>0.4086636480581222</v>
-      </c>
-      <c r="F8" s="69" t="n">
-        <v>0.3710155007741043</v>
-      </c>
-      <c r="G8" s="69" t="n">
-        <v>0.3740693678369545</v>
-      </c>
-      <c r="H8" s="69" t="n">
-        <v>0.3665146064743118</v>
-      </c>
-      <c r="I8" s="69" t="n">
-        <v>0.3160774852233587</v>
-      </c>
-      <c r="J8" s="69" t="n">
-        <v>0.2834731739911558</v>
-      </c>
-      <c r="K8" s="69" t="n">
-        <v>0.2681422535657876</v>
-      </c>
-      <c r="L8" s="69" t="n">
-        <v>0.2293236143202949</v>
-      </c>
-      <c r="M8" s="69" t="n">
-        <v>0.2237103228438481</v>
-      </c>
-      <c r="N8" s="69" t="n">
-        <v>0.2442902861034774</v>
-      </c>
-      <c r="O8" s="69" t="n">
-        <v>0.2543483353706967</v>
-      </c>
-      <c r="P8" s="69" t="n">
-        <v>0.2289710921190028</v>
-      </c>
-      <c r="Q8" s="69" t="n">
-        <v>0.1639623987109049</v>
-      </c>
-      <c r="R8" s="69" t="n">
-        <v>0.1637801712085247</v>
-      </c>
-      <c r="S8" s="69" t="n">
-        <v>0.1641121949179748</v>
-      </c>
-      <c r="T8" s="69" t="n">
-        <v>0.1502131462366411</v>
-      </c>
-      <c r="U8" s="69" t="n">
-        <v>0.1476627549294869</v>
-      </c>
-      <c r="V8" s="69" t="n">
-        <v>0.1493314823247189</v>
+      <c r="A8" s="70" t="inlineStr">
+        <is>
+          <t>Head of Research</t>
+        </is>
+      </c>
+      <c r="B8" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="71" t="n">
+        <v>0.05617977528089887</v>
+      </c>
+      <c r="D8" s="71" t="n">
+        <v>0.09316770186335403</v>
+      </c>
+      <c r="E8" s="71" t="n">
+        <v>0.078125</v>
+      </c>
+      <c r="F8" s="71" t="n">
+        <v>0.06726457399103139</v>
+      </c>
+      <c r="G8" s="71" t="n">
+        <v>0.06457167455876023</v>
+      </c>
+      <c r="H8" s="71" t="n">
+        <v>0.06208609271523179</v>
+      </c>
+      <c r="I8" s="71" t="n">
+        <v>0.05978477481068155</v>
+      </c>
+      <c r="J8" s="71" t="n">
+        <v>0.0576479631053036</v>
+      </c>
+      <c r="K8" s="71" t="n">
+        <v>0.05565862708719851</v>
+      </c>
+      <c r="L8" s="71" t="n">
+        <v>0.05410279531109107</v>
+      </c>
+      <c r="M8" s="71" t="n">
+        <v>0.05263157894736842</v>
+      </c>
+      <c r="N8" s="71" t="n">
+        <v>0.05123825789923143</v>
+      </c>
+      <c r="O8" s="71" t="n">
+        <v>0.04991680532445923</v>
+      </c>
+      <c r="P8" s="71" t="n">
+        <v>0.04866180048661801</v>
+      </c>
+      <c r="Q8" s="71" t="n">
+        <v>0.04746835443037975</v>
+      </c>
+      <c r="R8" s="71" t="n">
+        <v>0.04633204633204633</v>
+      </c>
+      <c r="S8" s="71" t="n">
+        <v>0.04524886877828054</v>
+      </c>
+      <c r="T8" s="71" t="n">
+        <v>0.04421518054532056</v>
+      </c>
+      <c r="U8" s="71" t="n">
+        <v>0.04322766570605188</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="70" t="inlineStr">
-        <is>
-          <t>Partner / Co-PM</t>
-        </is>
-      </c>
-      <c r="B9" s="71" t="n">
-        <v>0.243531202435312</v>
-      </c>
-      <c r="C9" s="71" t="n">
-        <v>0.250866141485368</v>
-      </c>
-      <c r="D9" s="71" t="n">
-        <v>0.2830188679245283</v>
-      </c>
-      <c r="E9" s="71" t="n">
-        <v>0.2451981888348733</v>
-      </c>
-      <c r="F9" s="71" t="n">
-        <v>0.2226093004644626</v>
-      </c>
-      <c r="G9" s="71" t="n">
-        <v>0.2244416207021727</v>
-      </c>
-      <c r="H9" s="71" t="n">
-        <v>0.2199087638845871</v>
-      </c>
-      <c r="I9" s="71" t="n">
-        <v>0.1896464911340152</v>
-      </c>
-      <c r="J9" s="71" t="n">
-        <v>0.2122853784665377</v>
-      </c>
-      <c r="K9" s="71" t="n">
-        <v>0.2269733893256809</v>
-      </c>
-      <c r="L9" s="71" t="n">
-        <v>0.2641641501512013</v>
-      </c>
-      <c r="M9" s="71" t="n">
-        <v>0.2684523874126177</v>
-      </c>
-      <c r="N9" s="71" t="n">
-        <v>0.2498251129911846</v>
-      </c>
-      <c r="O9" s="71" t="n">
-        <v>0.2401888528867841</v>
-      </c>
-      <c r="P9" s="71" t="n">
-        <v>0.2645018891634069</v>
-      </c>
-      <c r="Q9" s="71" t="n">
-        <v>0.241752041400785</v>
-      </c>
-      <c r="R9" s="71" t="n">
-        <v>0.2419135772641852</v>
-      </c>
-      <c r="S9" s="71" t="n">
-        <v>0.241619254311421</v>
-      </c>
-      <c r="T9" s="71" t="n">
-        <v>0.2539400884328099</v>
-      </c>
-      <c r="U9" s="71" t="n">
-        <v>0.256200886920571</v>
-      </c>
-      <c r="V9" s="71" t="n">
-        <v>0.2547216408295717</v>
+      <c r="A9" s="68" t="inlineStr">
+        <is>
+          <t>Senior Analyst</t>
+        </is>
+      </c>
+      <c r="B9" s="69" t="n">
+        <v>0.09433962264150944</v>
+      </c>
+      <c r="C9" s="69" t="n">
+        <v>0.0749063670411985</v>
+      </c>
+      <c r="D9" s="69" t="n">
+        <v>0.06211180124223602</v>
+      </c>
+      <c r="E9" s="69" t="n">
+        <v>0.078125</v>
+      </c>
+      <c r="F9" s="69" t="n">
+        <v>0.08968609865470852</v>
+      </c>
+      <c r="G9" s="69" t="n">
+        <v>0.09470512268618167</v>
+      </c>
+      <c r="H9" s="69" t="n">
+        <v>0.09933774834437087</v>
+      </c>
+      <c r="I9" s="69" t="n">
+        <v>0.1036269430051813</v>
+      </c>
+      <c r="J9" s="69" t="n">
+        <v>0.1076095311299001</v>
+      </c>
+      <c r="K9" s="69" t="n">
+        <v>0.111317254174397</v>
+      </c>
+      <c r="L9" s="69" t="n">
+        <v>0.1118124436429215</v>
+      </c>
+      <c r="M9" s="69" t="n">
+        <v>0.112280701754386</v>
+      </c>
+      <c r="N9" s="69" t="n">
+        <v>0.1127241673783091</v>
+      </c>
+      <c r="O9" s="69" t="n">
+        <v>0.1131447587354409</v>
+      </c>
+      <c r="P9" s="69" t="n">
+        <v>0.113544201135442</v>
+      </c>
+      <c r="Q9" s="69" t="n">
+        <v>0.1139240506329114</v>
+      </c>
+      <c r="R9" s="69" t="n">
+        <v>0.1142857142857143</v>
+      </c>
+      <c r="S9" s="69" t="n">
+        <v>0.114630467571644</v>
+      </c>
+      <c r="T9" s="69" t="n">
+        <v>0.1149594694178335</v>
+      </c>
+      <c r="U9" s="69" t="n">
+        <v>0.1152737752161383</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="68" t="inlineStr">
-        <is>
-          <t>Portfolio Manager</t>
-        </is>
-      </c>
-      <c r="B10" s="69" t="n">
-        <v>0.05073566717402334</v>
-      </c>
-      <c r="C10" s="69" t="n">
-        <v>0.04131138184910298</v>
-      </c>
-      <c r="D10" s="69" t="n">
+      <c r="A10" s="70" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="B10" s="71" t="n">
+        <v>0.05660377358490566</v>
+      </c>
+      <c r="C10" s="71" t="n">
+        <v>0.06741573033707865</v>
+      </c>
+      <c r="D10" s="71" t="n">
+        <v>0.07453416149068323</v>
+      </c>
+      <c r="E10" s="71" t="n">
+        <v>0.078125</v>
+      </c>
+      <c r="F10" s="71" t="n">
+        <v>0.08071748878923767</v>
+      </c>
+      <c r="G10" s="71" t="n">
+        <v>0.0826517434352131</v>
+      </c>
+      <c r="H10" s="71" t="n">
+        <v>0.08443708609271523</v>
+      </c>
+      <c r="I10" s="71" t="n">
+        <v>0.08609007572738143</v>
+      </c>
+      <c r="J10" s="71" t="n">
+        <v>0.08762490392006146</v>
+      </c>
+      <c r="K10" s="71" t="n">
+        <v>0.08905380333951762</v>
+      </c>
+      <c r="L10" s="71" t="n">
+        <v>0.09089269612263301</v>
+      </c>
+      <c r="M10" s="71" t="n">
+        <v>0.09263157894736843</v>
+      </c>
+      <c r="N10" s="71" t="n">
+        <v>0.09427839453458582</v>
+      </c>
+      <c r="O10" s="71" t="n">
+        <v>0.09584026622296173</v>
+      </c>
+      <c r="P10" s="71" t="n">
+        <v>0.09732360097323602</v>
+      </c>
+      <c r="Q10" s="71" t="n">
+        <v>0.09873417721518989</v>
+      </c>
+      <c r="R10" s="71" t="n">
+        <v>0.1000772200772201</v>
+      </c>
+      <c r="S10" s="71" t="n">
+        <v>0.1013574660633484</v>
+      </c>
+      <c r="T10" s="71" t="n">
+        <v>0.1025792188651437</v>
+      </c>
+      <c r="U10" s="71" t="n">
+        <v>0.1037463976945245</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="68" t="inlineStr">
+        <is>
+          <t>Junior Analyst</t>
+        </is>
+      </c>
+      <c r="B11" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="69" t="n">
-        <v>0.04859384222428394</v>
-      </c>
-      <c r="F10" s="69" t="n">
-        <v>0.07761714122141777</v>
-      </c>
-      <c r="G10" s="69" t="n">
-        <v>0.07526288734023868</v>
-      </c>
-      <c r="H10" s="69" t="n">
-        <v>0.08108692155434877</v>
-      </c>
-      <c r="I10" s="69" t="n">
-        <v>0.1199693568459926</v>
-      </c>
-      <c r="J10" s="69" t="n">
-        <v>0.1133892695964623</v>
-      </c>
-      <c r="K10" s="69" t="n">
-        <v>0.107256901426315</v>
-      </c>
-      <c r="L10" s="69" t="n">
-        <v>0.09172944572811798</v>
-      </c>
-      <c r="M10" s="69" t="n">
-        <v>0.09045271413385651</v>
-      </c>
-      <c r="N10" s="69" t="n">
-        <v>0.09771611444139094</v>
-      </c>
-      <c r="O10" s="69" t="n">
-        <v>0.1017393341482787</v>
-      </c>
-      <c r="P10" s="69" t="n">
-        <v>0.09158843684760112</v>
-      </c>
-      <c r="Q10" s="69" t="n">
-        <v>0.1611680276005233</v>
-      </c>
-      <c r="R10" s="69" t="n">
-        <v>0.1612757181761235</v>
-      </c>
-      <c r="S10" s="69" t="n">
-        <v>0.1610795028742807</v>
-      </c>
-      <c r="T10" s="69" t="n">
-        <v>0.1692933922885399</v>
-      </c>
-      <c r="U10" s="69" t="n">
-        <v>0.1708005912803806</v>
-      </c>
-      <c r="V10" s="69" t="n">
-        <v>0.1698144272197145</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="70" t="inlineStr">
-        <is>
-          <t>Head of Research</t>
-        </is>
-      </c>
-      <c r="B11" s="71" t="n">
-        <v>0.0380517503805175</v>
-      </c>
-      <c r="C11" s="71" t="n">
-        <v>0.03098353638682724</v>
-      </c>
-      <c r="D11" s="71" t="n">
+      <c r="C11" s="69" t="n">
+        <v>0.01123595505617977</v>
+      </c>
+      <c r="D11" s="69" t="n">
+        <v>0.01863354037267081</v>
+      </c>
+      <c r="E11" s="69" t="n">
+        <v>0.0234375</v>
+      </c>
+      <c r="F11" s="69" t="n">
+        <v>0.02690582959641256</v>
+      </c>
+      <c r="G11" s="69" t="n">
+        <v>0.0284115368058545</v>
+      </c>
+      <c r="H11" s="69" t="n">
+        <v>0.02980132450331125</v>
+      </c>
+      <c r="I11" s="69" t="n">
+        <v>0.03108808290155441</v>
+      </c>
+      <c r="J11" s="69" t="n">
+        <v>0.03228285933897001</v>
+      </c>
+      <c r="K11" s="69" t="n">
+        <v>0.03339517625231911</v>
+      </c>
+      <c r="L11" s="69" t="n">
+        <v>0.03354373309287647</v>
+      </c>
+      <c r="M11" s="69" t="n">
+        <v>0.0336842105263158</v>
+      </c>
+      <c r="N11" s="69" t="n">
+        <v>0.03381725021349274</v>
+      </c>
+      <c r="O11" s="69" t="n">
+        <v>0.03394342762063228</v>
+      </c>
+      <c r="P11" s="69" t="n">
+        <v>0.0340632603406326</v>
+      </c>
+      <c r="Q11" s="69" t="n">
+        <v>0.03417721518987342</v>
+      </c>
+      <c r="R11" s="69" t="n">
+        <v>0.03428571428571429</v>
+      </c>
+      <c r="S11" s="69" t="n">
+        <v>0.03438914027149321</v>
+      </c>
+      <c r="T11" s="69" t="n">
+        <v>0.03448784082535004</v>
+      </c>
+      <c r="U11" s="69" t="n">
+        <v>0.0345821325648415</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="70" t="inlineStr">
+        <is>
+          <t>Head of Trading</t>
+        </is>
+      </c>
+      <c r="B12" s="71" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="71" t="n">
-        <v>0.03644538166821296</v>
-      </c>
-      <c r="F11" s="71" t="n">
-        <v>0.05821285591606334</v>
-      </c>
-      <c r="G11" s="71" t="n">
-        <v>0.05644716550517902</v>
-      </c>
-      <c r="H11" s="71" t="n">
-        <v>0.06081519116576158</v>
-      </c>
-      <c r="I11" s="71" t="n">
-        <v>0.08997701763449445</v>
-      </c>
-      <c r="J11" s="71" t="n">
-        <v>0.08504195219734675</v>
-      </c>
-      <c r="K11" s="71" t="n">
-        <v>0.08044267606973626</v>
-      </c>
-      <c r="L11" s="71" t="n">
-        <v>0.06879708429608848</v>
-      </c>
-      <c r="M11" s="71" t="n">
-        <v>0.06711309685315443</v>
-      </c>
-      <c r="N11" s="71" t="n">
-        <v>0.07328708583104321</v>
-      </c>
-      <c r="O11" s="71" t="n">
-        <v>0.07630450061120903</v>
-      </c>
-      <c r="P11" s="71" t="n">
-        <v>0.06869132763570084</v>
-      </c>
-      <c r="Q11" s="71" t="n">
-        <v>0.04918871961327147</v>
-      </c>
-      <c r="R11" s="71" t="n">
-        <v>0.04913405136255741</v>
-      </c>
-      <c r="S11" s="71" t="n">
-        <v>0.04923365847539245</v>
-      </c>
-      <c r="T11" s="71" t="n">
-        <v>0.04506394387099233</v>
-      </c>
-      <c r="U11" s="71" t="n">
-        <v>0.04429882647884606</v>
-      </c>
-      <c r="V11" s="71" t="n">
-        <v>0.04479944469741567</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="68" t="inlineStr">
-        <is>
-          <t>Senior Analyst</t>
-        </is>
-      </c>
-      <c r="B12" s="69" t="n">
-        <v>0.08117706747843734</v>
-      </c>
-      <c r="C12" s="69" t="n">
-        <v>0.08362204716178932</v>
-      </c>
-      <c r="D12" s="69" t="n">
-        <v>0.09433962264150944</v>
-      </c>
-      <c r="E12" s="69" t="n">
-        <v>0.08173272961162445</v>
-      </c>
-      <c r="F12" s="69" t="n">
-        <v>0.07420310015482087</v>
-      </c>
-      <c r="G12" s="69" t="n">
-        <v>0.07481387356739091</v>
-      </c>
-      <c r="H12" s="69" t="n">
-        <v>0.07330292129486236</v>
-      </c>
-      <c r="I12" s="69" t="n">
-        <v>0.06321549704467173</v>
-      </c>
-      <c r="J12" s="69" t="n">
-        <v>0.07076179282217923</v>
-      </c>
-      <c r="K12" s="69" t="n">
-        <v>0.07565779644189363</v>
-      </c>
-      <c r="L12" s="69" t="n">
-        <v>0.08805471671706708</v>
-      </c>
-      <c r="M12" s="69" t="n">
-        <v>0.08996842163569788</v>
-      </c>
-      <c r="N12" s="69" t="n">
-        <v>0.08327503766372819</v>
-      </c>
-      <c r="O12" s="69" t="n">
-        <v>0.08006295096226136</v>
-      </c>
-      <c r="P12" s="69" t="n">
-        <v>0.08816729638780231</v>
-      </c>
-      <c r="Q12" s="69" t="n">
-        <v>0.1133764935424426</v>
-      </c>
-      <c r="R12" s="69" t="n">
-        <v>0.1133938933297667</v>
-      </c>
-      <c r="S12" s="69" t="n">
-        <v>0.1133621904207353</v>
-      </c>
-      <c r="T12" s="69" t="n">
-        <v>0.1146893253915982</v>
-      </c>
-      <c r="U12" s="69" t="n">
-        <v>0.1149328466260877</v>
-      </c>
-      <c r="V12" s="69" t="n">
-        <v>0.114773510074801</v>
+      <c r="C12" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="71" t="n">
+        <v>0.0234375</v>
+      </c>
+      <c r="F12" s="71" t="n">
+        <v>0.04035874439461883</v>
+      </c>
+      <c r="G12" s="71" t="n">
+        <v>0.03874300473525614</v>
+      </c>
+      <c r="H12" s="71" t="n">
+        <v>0.03725165562913908</v>
+      </c>
+      <c r="I12" s="71" t="n">
+        <v>0.03587086488640893</v>
+      </c>
+      <c r="J12" s="71" t="n">
+        <v>0.03458877786318216</v>
+      </c>
+      <c r="K12" s="71" t="n">
+        <v>0.03339517625231911</v>
+      </c>
+      <c r="L12" s="71" t="n">
+        <v>0.03246167718665464</v>
+      </c>
+      <c r="M12" s="71" t="n">
+        <v>0.03157894736842105</v>
+      </c>
+      <c r="N12" s="71" t="n">
+        <v>0.03074295473953886</v>
+      </c>
+      <c r="O12" s="71" t="n">
+        <v>0.02995008319467554</v>
+      </c>
+      <c r="P12" s="71" t="n">
+        <v>0.0291970802919708</v>
+      </c>
+      <c r="Q12" s="71" t="n">
+        <v>0.02848101265822785</v>
+      </c>
+      <c r="R12" s="71" t="n">
+        <v>0.0277992277992278</v>
+      </c>
+      <c r="S12" s="71" t="n">
+        <v>0.02714932126696833</v>
+      </c>
+      <c r="T12" s="71" t="n">
+        <v>0.02652910832719233</v>
+      </c>
+      <c r="U12" s="71" t="n">
+        <v>0.02593659942363112</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="70" t="inlineStr">
-        <is>
-          <t>Analyst</t>
-        </is>
-      </c>
-      <c r="B13" s="71" t="n">
-        <v>0.0639269406392694</v>
-      </c>
-      <c r="C13" s="71" t="n">
-        <v>0.06256664285180449</v>
-      </c>
-      <c r="D13" s="71" t="n">
-        <v>0.05660377358490566</v>
-      </c>
-      <c r="E13" s="71" t="n">
-        <v>0.06361779043425984</v>
-      </c>
-      <c r="F13" s="71" t="n">
-        <v>0.06780700245931787</v>
-      </c>
-      <c r="G13" s="71" t="n">
-        <v>0.06746719034250616</v>
-      </c>
-      <c r="H13" s="71" t="n">
-        <v>0.06830782924322205</v>
-      </c>
-      <c r="I13" s="71" t="n">
-        <v>0.07392010528060082</v>
-      </c>
-      <c r="J13" s="71" t="n">
-        <v>0.07647385657224623</v>
-      </c>
-      <c r="K13" s="71" t="n">
-        <v>0.07757174829303069</v>
-      </c>
-      <c r="L13" s="71" t="n">
-        <v>0.08035166374867565</v>
-      </c>
-      <c r="M13" s="71" t="n">
-        <v>0.08082629172268051</v>
-      </c>
-      <c r="N13" s="71" t="n">
-        <v>0.0792798569306542</v>
-      </c>
-      <c r="O13" s="71" t="n">
-        <v>0.07855957082184042</v>
-      </c>
-      <c r="P13" s="71" t="n">
-        <v>0.08037690888696172</v>
-      </c>
-      <c r="Q13" s="71" t="n">
-        <v>0.096700816560314</v>
-      </c>
-      <c r="R13" s="71" t="n">
-        <v>0.09676543090567409</v>
-      </c>
-      <c r="S13" s="71" t="n">
-        <v>0.09664770172456839</v>
-      </c>
-      <c r="T13" s="71" t="n">
-        <v>0.1015760353731239</v>
-      </c>
-      <c r="U13" s="71" t="n">
-        <v>0.1024803547682284</v>
-      </c>
-      <c r="V13" s="71" t="n">
-        <v>0.1018886563318287</v>
+      <c r="A13" s="68" t="inlineStr">
+        <is>
+          <t>Trader / Execution</t>
+        </is>
+      </c>
+      <c r="B13" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="69" t="n">
+        <v>0.01872659176029963</v>
+      </c>
+      <c r="D13" s="69" t="n">
+        <v>0.03105590062111801</v>
+      </c>
+      <c r="E13" s="69" t="n">
+        <v>0.02604166666666667</v>
+      </c>
+      <c r="F13" s="69" t="n">
+        <v>0.02242152466367713</v>
+      </c>
+      <c r="G13" s="69" t="n">
+        <v>0.02582866982350409</v>
+      </c>
+      <c r="H13" s="69" t="n">
+        <v>0.02897350993377484</v>
+      </c>
+      <c r="I13" s="69" t="n">
+        <v>0.03188521323236349</v>
+      </c>
+      <c r="J13" s="69" t="n">
+        <v>0.03458877786318216</v>
+      </c>
+      <c r="K13" s="69" t="n">
+        <v>0.03710575139146568</v>
+      </c>
+      <c r="L13" s="69" t="n">
+        <v>0.03606853020739405</v>
+      </c>
+      <c r="M13" s="69" t="n">
+        <v>0.03508771929824561</v>
+      </c>
+      <c r="N13" s="69" t="n">
+        <v>0.03415883859948762</v>
+      </c>
+      <c r="O13" s="69" t="n">
+        <v>0.03327787021630615</v>
+      </c>
+      <c r="P13" s="69" t="n">
+        <v>0.032441200324412</v>
+      </c>
+      <c r="Q13" s="69" t="n">
+        <v>0.03164556962025317</v>
+      </c>
+      <c r="R13" s="69" t="n">
+        <v>0.03088803088803089</v>
+      </c>
+      <c r="S13" s="69" t="n">
+        <v>0.0301659125188537</v>
+      </c>
+      <c r="T13" s="69" t="n">
+        <v>0.02947678703021371</v>
+      </c>
+      <c r="U13" s="69" t="n">
+        <v>0.02881844380403458</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="68" t="inlineStr">
-        <is>
-          <t>Junior Analyst</t>
-        </is>
-      </c>
-      <c r="B14" s="69" t="n">
-        <v>0.0076103500761035</v>
-      </c>
-      <c r="C14" s="69" t="n">
-        <v>0.006196707277365446</v>
-      </c>
-      <c r="D14" s="69" t="n">
+      <c r="A14" s="70" t="inlineStr">
+        <is>
+          <t>COO / Head of Operations</t>
+        </is>
+      </c>
+      <c r="B14" s="71" t="n">
+        <v>0.07075471698113207</v>
+      </c>
+      <c r="C14" s="71" t="n">
+        <v>0.05617977528089887</v>
+      </c>
+      <c r="D14" s="71" t="n">
+        <v>0.04658385093167702</v>
+      </c>
+      <c r="E14" s="71" t="n">
+        <v>0.0390625</v>
+      </c>
+      <c r="F14" s="71" t="n">
+        <v>0.0336322869955157</v>
+      </c>
+      <c r="G14" s="71" t="n">
+        <v>0.03228583727938011</v>
+      </c>
+      <c r="H14" s="71" t="n">
+        <v>0.0310430463576159</v>
+      </c>
+      <c r="I14" s="71" t="n">
+        <v>0.02989238740534077</v>
+      </c>
+      <c r="J14" s="71" t="n">
+        <v>0.0288239815526518</v>
+      </c>
+      <c r="K14" s="71" t="n">
+        <v>0.02782931354359926</v>
+      </c>
+      <c r="L14" s="71" t="n">
+        <v>0.02705139765554554</v>
+      </c>
+      <c r="M14" s="71" t="n">
+        <v>0.02631578947368421</v>
+      </c>
+      <c r="N14" s="71" t="n">
+        <v>0.02561912894961571</v>
+      </c>
+      <c r="O14" s="71" t="n">
+        <v>0.02495840266222962</v>
+      </c>
+      <c r="P14" s="71" t="n">
+        <v>0.024330900243309</v>
+      </c>
+      <c r="Q14" s="71" t="n">
+        <v>0.02373417721518987</v>
+      </c>
+      <c r="R14" s="71" t="n">
+        <v>0.02316602316602316</v>
+      </c>
+      <c r="S14" s="71" t="n">
+        <v>0.02262443438914027</v>
+      </c>
+      <c r="T14" s="71" t="n">
+        <v>0.02210759027266028</v>
+      </c>
+      <c r="U14" s="71" t="n">
+        <v>0.02161383285302594</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="68" t="inlineStr">
+        <is>
+          <t>CFO / Finance</t>
+        </is>
+      </c>
+      <c r="B15" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="69" t="n">
-        <v>0.007289076333642593</v>
-      </c>
-      <c r="F14" s="69" t="n">
-        <v>0.01164257118321267</v>
-      </c>
-      <c r="G14" s="69" t="n">
-        <v>0.0112894331010358</v>
-      </c>
-      <c r="H14" s="69" t="n">
-        <v>0.01216303823315231</v>
-      </c>
-      <c r="I14" s="69" t="n">
-        <v>0.01799540352689889</v>
-      </c>
-      <c r="J14" s="69" t="n">
-        <v>0.02122853784665377</v>
-      </c>
-      <c r="K14" s="69" t="n">
-        <v>0.02269733893256809</v>
-      </c>
-      <c r="L14" s="69" t="n">
-        <v>0.02641641501512013</v>
-      </c>
-      <c r="M14" s="69" t="n">
-        <v>0.02699052649070936</v>
-      </c>
-      <c r="N14" s="69" t="n">
-        <v>0.02498251129911846</v>
-      </c>
-      <c r="O14" s="69" t="n">
-        <v>0.02401888528867841</v>
-      </c>
-      <c r="P14" s="69" t="n">
-        <v>0.02645018891634069</v>
-      </c>
-      <c r="Q14" s="69" t="n">
-        <v>0.03401294806273279</v>
-      </c>
-      <c r="R14" s="69" t="n">
-        <v>0.03401816799893</v>
-      </c>
-      <c r="S14" s="69" t="n">
-        <v>0.03400865712622059</v>
-      </c>
-      <c r="T14" s="69" t="n">
-        <v>0.03440679761747945</v>
-      </c>
-      <c r="U14" s="69" t="n">
-        <v>0.03447985398782631</v>
-      </c>
-      <c r="V14" s="69" t="n">
-        <v>0.0344320530224403</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="70" t="inlineStr">
-        <is>
-          <t>Head of Trading</t>
-        </is>
-      </c>
-      <c r="B15" s="71" t="n">
+      <c r="C15" s="69" t="n">
+        <v>0.02247191011235955</v>
+      </c>
+      <c r="D15" s="69" t="n">
+        <v>0.03726708074534162</v>
+      </c>
+      <c r="E15" s="69" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="F15" s="69" t="n">
+        <v>0.02690582959641256</v>
+      </c>
+      <c r="G15" s="69" t="n">
+        <v>0.02582866982350409</v>
+      </c>
+      <c r="H15" s="69" t="n">
+        <v>0.02483443708609272</v>
+      </c>
+      <c r="I15" s="69" t="n">
+        <v>0.02391390992427262</v>
+      </c>
+      <c r="J15" s="69" t="n">
+        <v>0.02305918524212144</v>
+      </c>
+      <c r="K15" s="69" t="n">
+        <v>0.02226345083487941</v>
+      </c>
+      <c r="L15" s="69" t="n">
+        <v>0.02164111812443643</v>
+      </c>
+      <c r="M15" s="69" t="n">
+        <v>0.02105263157894737</v>
+      </c>
+      <c r="N15" s="69" t="n">
+        <v>0.02049530315969257</v>
+      </c>
+      <c r="O15" s="69" t="n">
+        <v>0.01996672212978369</v>
+      </c>
+      <c r="P15" s="69" t="n">
+        <v>0.0194647201946472</v>
+      </c>
+      <c r="Q15" s="69" t="n">
+        <v>0.0189873417721519</v>
+      </c>
+      <c r="R15" s="69" t="n">
+        <v>0.01853281853281853</v>
+      </c>
+      <c r="S15" s="69" t="n">
+        <v>0.01809954751131222</v>
+      </c>
+      <c r="T15" s="69" t="n">
+        <v>0.01768607221812822</v>
+      </c>
+      <c r="U15" s="69" t="n">
+        <v>0.01729106628242075</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="70" t="inlineStr">
+        <is>
+          <t>Compliance / Legal</t>
+        </is>
+      </c>
+      <c r="B16" s="71" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="71" t="n">
+      <c r="C16" s="71" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="71" t="n">
+      <c r="D16" s="71" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="71" t="n">
-        <v>0.01266044222155325</v>
-      </c>
-      <c r="K15" s="71" t="n">
-        <v>0.01982641115586252</v>
-      </c>
-      <c r="L15" s="71" t="n">
-        <v>0.03797099446770729</v>
-      </c>
-      <c r="M15" s="71" t="n">
-        <v>0.04026785811189266</v>
-      </c>
-      <c r="N15" s="71" t="n">
-        <v>0.03097528239872945</v>
-      </c>
-      <c r="O15" s="71" t="n">
-        <v>0.02627395549930982</v>
-      </c>
-      <c r="P15" s="71" t="n">
-        <v>0.03813577016760158</v>
-      </c>
-      <c r="Q15" s="71" t="n">
-        <v>0.02951323176796288</v>
-      </c>
-      <c r="R15" s="71" t="n">
-        <v>0.02948043081753444</v>
-      </c>
-      <c r="S15" s="71" t="n">
-        <v>0.02954019508523547</v>
-      </c>
-      <c r="T15" s="71" t="n">
-        <v>0.0270383663225954</v>
-      </c>
-      <c r="U15" s="71" t="n">
-        <v>0.02657929588730763</v>
-      </c>
-      <c r="V15" s="71" t="n">
-        <v>0.02687966681844941</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="68" t="inlineStr">
-        <is>
-          <t>Trader / Execution</t>
-        </is>
-      </c>
-      <c r="B16" s="69" t="n">
-        <v>0.01268391679350583</v>
-      </c>
-      <c r="C16" s="69" t="n">
-        <v>0.01032784546227574</v>
-      </c>
-      <c r="D16" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="69" t="n">
-        <v>0.01214846055607099</v>
-      </c>
-      <c r="F16" s="69" t="n">
-        <v>0.01940428530535444</v>
-      </c>
-      <c r="G16" s="69" t="n">
-        <v>0.01881572183505967</v>
-      </c>
-      <c r="H16" s="69" t="n">
-        <v>0.02027173038858719</v>
-      </c>
-      <c r="I16" s="69" t="n">
-        <v>0.02999233921149815</v>
-      </c>
-      <c r="J16" s="69" t="n">
-        <v>0.02834731739911558</v>
-      </c>
-      <c r="K16" s="69" t="n">
-        <v>0.02681422535657876</v>
-      </c>
-      <c r="L16" s="69" t="n">
-        <v>0.02293236143202949</v>
-      </c>
-      <c r="M16" s="69" t="n">
-        <v>0.02261317853346413</v>
-      </c>
-      <c r="N16" s="69" t="n">
-        <v>0.02442902861034774</v>
-      </c>
-      <c r="O16" s="69" t="n">
-        <v>0.02543483353706967</v>
-      </c>
-      <c r="P16" s="69" t="n">
-        <v>0.02289710921190028</v>
-      </c>
-      <c r="Q16" s="69" t="n">
-        <v>0.03279247974218098</v>
-      </c>
-      <c r="R16" s="69" t="n">
-        <v>0.03275603424170494</v>
-      </c>
-      <c r="S16" s="69" t="n">
-        <v>0.03282243898359496</v>
-      </c>
-      <c r="T16" s="69" t="n">
-        <v>0.03004262924732822</v>
-      </c>
-      <c r="U16" s="69" t="n">
-        <v>0.02953255098589737</v>
-      </c>
-      <c r="V16" s="69" t="n">
-        <v>0.02986629646494378</v>
+      <c r="E16" s="71" t="n">
+        <v>0.01041666666666667</v>
+      </c>
+      <c r="F16" s="71" t="n">
+        <v>0.0179372197309417</v>
+      </c>
+      <c r="G16" s="71" t="n">
+        <v>0.01721911321566939</v>
+      </c>
+      <c r="H16" s="71" t="n">
+        <v>0.01655629139072848</v>
+      </c>
+      <c r="I16" s="71" t="n">
+        <v>0.01594260661618175</v>
+      </c>
+      <c r="J16" s="71" t="n">
+        <v>0.01537279016141429</v>
+      </c>
+      <c r="K16" s="71" t="n">
+        <v>0.01484230055658627</v>
+      </c>
+      <c r="L16" s="71" t="n">
+        <v>0.01442741208295762</v>
+      </c>
+      <c r="M16" s="71" t="n">
+        <v>0.01403508771929825</v>
+      </c>
+      <c r="N16" s="71" t="n">
+        <v>0.01366353543979505</v>
+      </c>
+      <c r="O16" s="71" t="n">
+        <v>0.01331114808652246</v>
+      </c>
+      <c r="P16" s="71" t="n">
+        <v>0.0129764801297648</v>
+      </c>
+      <c r="Q16" s="71" t="n">
+        <v>0.01265822784810127</v>
+      </c>
+      <c r="R16" s="71" t="n">
+        <v>0.01235521235521236</v>
+      </c>
+      <c r="S16" s="71" t="n">
+        <v>0.01206636500754148</v>
+      </c>
+      <c r="T16" s="71" t="n">
+        <v>0.01179071481208548</v>
+      </c>
+      <c r="U16" s="71" t="n">
+        <v>0.01152737752161383</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="70" t="inlineStr">
-        <is>
-          <t>COO / Head of Operations</t>
-        </is>
-      </c>
-      <c r="B17" s="71" t="n">
-        <v>0.060882800608828</v>
-      </c>
-      <c r="C17" s="71" t="n">
-        <v>0.062716535371342</v>
-      </c>
-      <c r="D17" s="71" t="n">
-        <v>0.07075471698113207</v>
-      </c>
-      <c r="E17" s="71" t="n">
-        <v>0.06129954720871834</v>
-      </c>
-      <c r="F17" s="71" t="n">
-        <v>0.05565232511611565</v>
-      </c>
-      <c r="G17" s="71" t="n">
-        <v>0.05611040517554319</v>
-      </c>
-      <c r="H17" s="71" t="n">
-        <v>0.05497719097114678</v>
-      </c>
-      <c r="I17" s="71" t="n">
-        <v>0.0474116227835038</v>
-      </c>
-      <c r="J17" s="71" t="n">
-        <v>0.04252097609867338</v>
-      </c>
-      <c r="K17" s="71" t="n">
-        <v>0.04022133803486813</v>
-      </c>
-      <c r="L17" s="71" t="n">
-        <v>0.03439854214804424</v>
-      </c>
-      <c r="M17" s="71" t="n">
-        <v>0.03355654842657722</v>
-      </c>
-      <c r="N17" s="71" t="n">
-        <v>0.0366435429155216</v>
-      </c>
-      <c r="O17" s="71" t="n">
-        <v>0.03815225030560451</v>
-      </c>
-      <c r="P17" s="71" t="n">
-        <v>0.03434566381785042</v>
-      </c>
-      <c r="Q17" s="71" t="n">
-        <v>0.02459435980663573</v>
-      </c>
-      <c r="R17" s="71" t="n">
-        <v>0.0245670256812787</v>
-      </c>
-      <c r="S17" s="71" t="n">
-        <v>0.02461682923769622</v>
-      </c>
-      <c r="T17" s="71" t="n">
-        <v>0.02253197193549616</v>
-      </c>
-      <c r="U17" s="71" t="n">
-        <v>0.02214941323942303</v>
-      </c>
-      <c r="V17" s="71" t="n">
-        <v>0.02239972234870784</v>
+      <c r="A17" s="68" t="inlineStr">
+        <is>
+          <t>Investor Relations / Ops</t>
+        </is>
+      </c>
+      <c r="B17" s="69" t="n">
+        <v>0.02358490566037736</v>
+      </c>
+      <c r="C17" s="69" t="n">
+        <v>0.01872659176029963</v>
+      </c>
+      <c r="D17" s="69" t="n">
+        <v>0.01552795031055901</v>
+      </c>
+      <c r="E17" s="69" t="n">
+        <v>0.01302083333333333</v>
+      </c>
+      <c r="F17" s="69" t="n">
+        <v>0.01121076233183856</v>
+      </c>
+      <c r="G17" s="69" t="n">
+        <v>0.01291433491175204</v>
+      </c>
+      <c r="H17" s="69" t="n">
+        <v>0.01448675496688742</v>
+      </c>
+      <c r="I17" s="69" t="n">
+        <v>0.01594260661618175</v>
+      </c>
+      <c r="J17" s="69" t="n">
+        <v>0.01729438893159108</v>
+      </c>
+      <c r="K17" s="69" t="n">
+        <v>0.01855287569573284</v>
+      </c>
+      <c r="L17" s="69" t="n">
+        <v>0.01893597835888187</v>
+      </c>
+      <c r="M17" s="69" t="n">
+        <v>0.01929824561403509</v>
+      </c>
+      <c r="N17" s="69" t="n">
+        <v>0.01964133219470538</v>
+      </c>
+      <c r="O17" s="69" t="n">
+        <v>0.01996672212978369</v>
+      </c>
+      <c r="P17" s="69" t="n">
+        <v>0.0202757502027575</v>
+      </c>
+      <c r="Q17" s="69" t="n">
+        <v>0.02056962025316456</v>
+      </c>
+      <c r="R17" s="69" t="n">
+        <v>0.02084942084942085</v>
+      </c>
+      <c r="S17" s="69" t="n">
+        <v>0.02111613876319759</v>
+      </c>
+      <c r="T17" s="69" t="n">
+        <v>0.02137067059690494</v>
+      </c>
+      <c r="U17" s="69" t="n">
+        <v>0.02161383285302594</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="68" t="inlineStr">
-        <is>
-          <t>CFO / Finance</t>
-        </is>
-      </c>
-      <c r="B18" s="69" t="n">
-        <v>0.015220700152207</v>
-      </c>
-      <c r="C18" s="69" t="n">
-        <v>0.01239341455473089</v>
-      </c>
-      <c r="D18" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="69" t="n">
-        <v>0.01457815266728519</v>
-      </c>
-      <c r="F18" s="69" t="n">
-        <v>0.02328514236642533</v>
-      </c>
-      <c r="G18" s="69" t="n">
-        <v>0.02257886620207161</v>
-      </c>
-      <c r="H18" s="69" t="n">
-        <v>0.02432607646630463</v>
-      </c>
-      <c r="I18" s="69" t="n">
-        <v>0.03599080705379777</v>
-      </c>
-      <c r="J18" s="69" t="n">
-        <v>0.0340167808789387</v>
-      </c>
-      <c r="K18" s="69" t="n">
-        <v>0.03217707042789451</v>
-      </c>
-      <c r="L18" s="69" t="n">
-        <v>0.02751883371843539</v>
-      </c>
-      <c r="M18" s="69" t="n">
-        <v>0.02684523874126177</v>
-      </c>
-      <c r="N18" s="69" t="n">
-        <v>0.02931483433241728</v>
-      </c>
-      <c r="O18" s="69" t="n">
-        <v>0.03052180024448361</v>
-      </c>
-      <c r="P18" s="69" t="n">
-        <v>0.02747653105428034</v>
-      </c>
-      <c r="Q18" s="69" t="n">
-        <v>0.01967548784530859</v>
-      </c>
-      <c r="R18" s="69" t="n">
-        <v>0.01965362054502296</v>
-      </c>
-      <c r="S18" s="69" t="n">
-        <v>0.01969346339015698</v>
-      </c>
-      <c r="T18" s="69" t="n">
-        <v>0.01802557754839693</v>
-      </c>
-      <c r="U18" s="69" t="n">
-        <v>0.01771953059153842</v>
-      </c>
-      <c r="V18" s="69" t="n">
-        <v>0.01791977787896627</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="70" t="inlineStr">
-        <is>
-          <t>Compliance / Legal</t>
-        </is>
-      </c>
-      <c r="B19" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="71" t="n">
-        <v>0.00562686320957922</v>
-      </c>
-      <c r="K19" s="71" t="n">
-        <v>0.008811738291494453</v>
-      </c>
-      <c r="L19" s="71" t="n">
-        <v>0.01687599754120324</v>
-      </c>
-      <c r="M19" s="71" t="n">
-        <v>0.01789682582750785</v>
-      </c>
-      <c r="N19" s="71" t="n">
-        <v>0.01376679217721309</v>
-      </c>
-      <c r="O19" s="71" t="n">
-        <v>0.01167731355524881</v>
-      </c>
-      <c r="P19" s="71" t="n">
-        <v>0.0169492311856007</v>
-      </c>
-      <c r="Q19" s="71" t="n">
-        <v>0.01311699189687239</v>
-      </c>
-      <c r="R19" s="71" t="n">
-        <v>0.01310241369668197</v>
-      </c>
-      <c r="S19" s="71" t="n">
-        <v>0.01312897559343799</v>
-      </c>
-      <c r="T19" s="71" t="n">
-        <v>0.01201705169893129</v>
-      </c>
-      <c r="U19" s="71" t="n">
-        <v>0.01181302039435895</v>
-      </c>
-      <c r="V19" s="71" t="n">
-        <v>0.01194651858597751</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="68" t="inlineStr">
-        <is>
-          <t>Investor Relations / Ops</t>
-        </is>
-      </c>
-      <c r="B20" s="69" t="n">
-        <v>0.02029426686960933</v>
-      </c>
-      <c r="C20" s="69" t="n">
-        <v>0.02090551179044733</v>
-      </c>
-      <c r="D20" s="69" t="n">
-        <v>0.02358490566037736</v>
-      </c>
-      <c r="E20" s="69" t="n">
-        <v>0.02043318240290611</v>
-      </c>
-      <c r="F20" s="69" t="n">
-        <v>0.01855077503870522</v>
-      </c>
-      <c r="G20" s="69" t="n">
-        <v>0.01870346839184773</v>
-      </c>
-      <c r="H20" s="69" t="n">
-        <v>0.01832573032371559</v>
-      </c>
-      <c r="I20" s="69" t="n">
-        <v>0.01580387426116793</v>
-      </c>
-      <c r="J20" s="69" t="n">
-        <v>0.01417365869955779</v>
-      </c>
-      <c r="K20" s="69" t="n">
-        <v>0.01340711267828938</v>
-      </c>
-      <c r="L20" s="69" t="n">
-        <v>0.01146618071601475</v>
-      </c>
-      <c r="M20" s="69" t="n">
-        <v>0.01130658926673206</v>
-      </c>
-      <c r="N20" s="69" t="n">
-        <v>0.01221451430517387</v>
-      </c>
-      <c r="O20" s="69" t="n">
-        <v>0.01271741676853484</v>
-      </c>
-      <c r="P20" s="69" t="n">
-        <v>0.01144855460595014</v>
-      </c>
-      <c r="Q20" s="69" t="n">
-        <v>0.02014600345006541</v>
-      </c>
-      <c r="R20" s="69" t="n">
-        <v>0.02015946477201543</v>
-      </c>
-      <c r="S20" s="69" t="n">
-        <v>0.02013493785928508</v>
-      </c>
-      <c r="T20" s="69" t="n">
-        <v>0.02116167403606749</v>
-      </c>
-      <c r="U20" s="69" t="n">
-        <v>0.02135007391004758</v>
-      </c>
-      <c r="V20" s="69" t="n">
-        <v>0.02122680340246431</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="72" t="inlineStr">
+      <c r="A18" s="72" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B21" s="73">
-        <f>SUM(B8:B20)</f>
-        <v/>
-      </c>
-      <c r="C21" s="73">
-        <f>SUM(C8:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="73">
-        <f>SUM(D8:D20)</f>
-        <v/>
-      </c>
-      <c r="E21" s="73">
-        <f>SUM(E8:E20)</f>
-        <v/>
-      </c>
-      <c r="F21" s="73">
-        <f>SUM(F8:F20)</f>
-        <v/>
-      </c>
-      <c r="G21" s="73">
-        <f>SUM(G8:G20)</f>
-        <v/>
-      </c>
-      <c r="H21" s="73">
-        <f>SUM(H8:H20)</f>
-        <v/>
-      </c>
-      <c r="I21" s="73">
-        <f>SUM(I8:I20)</f>
-        <v/>
-      </c>
-      <c r="J21" s="73">
-        <f>SUM(J8:J20)</f>
-        <v/>
-      </c>
-      <c r="K21" s="73">
-        <f>SUM(K8:K20)</f>
-        <v/>
-      </c>
-      <c r="L21" s="73">
-        <f>SUM(L8:L20)</f>
-        <v/>
-      </c>
-      <c r="M21" s="73">
-        <f>SUM(M8:M20)</f>
-        <v/>
-      </c>
-      <c r="N21" s="73">
-        <f>SUM(N8:N20)</f>
-        <v/>
-      </c>
-      <c r="O21" s="73">
-        <f>SUM(O8:O20)</f>
-        <v/>
-      </c>
-      <c r="P21" s="73">
-        <f>SUM(P8:P20)</f>
-        <v/>
-      </c>
-      <c r="Q21" s="73">
-        <f>SUM(Q8:Q20)</f>
-        <v/>
-      </c>
-      <c r="R21" s="73">
-        <f>SUM(R8:R20)</f>
-        <v/>
-      </c>
-      <c r="S21" s="73">
-        <f>SUM(S8:S20)</f>
-        <v/>
-      </c>
-      <c r="T21" s="73">
-        <f>SUM(T8:T20)</f>
-        <v/>
-      </c>
-      <c r="U21" s="73">
-        <f>SUM(U8:U20)</f>
-        <v/>
-      </c>
-      <c r="V21" s="73">
-        <f>SUM(V8:V20)</f>
+      <c r="B18" s="73">
+        <f>SUM(B5:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="73">
+        <f>SUM(C5:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="73">
+        <f>SUM(D5:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="73">
+        <f>SUM(E5:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="73">
+        <f>SUM(F5:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="73">
+        <f>SUM(G5:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="73">
+        <f>SUM(H5:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="73">
+        <f>SUM(I5:I17)</f>
+        <v/>
+      </c>
+      <c r="J18" s="73">
+        <f>SUM(J5:J17)</f>
+        <v/>
+      </c>
+      <c r="K18" s="73">
+        <f>SUM(K5:K17)</f>
+        <v/>
+      </c>
+      <c r="L18" s="73">
+        <f>SUM(L5:L17)</f>
+        <v/>
+      </c>
+      <c r="M18" s="73">
+        <f>SUM(M5:M17)</f>
+        <v/>
+      </c>
+      <c r="N18" s="73">
+        <f>SUM(N5:N17)</f>
+        <v/>
+      </c>
+      <c r="O18" s="73">
+        <f>SUM(O5:O17)</f>
+        <v/>
+      </c>
+      <c r="P18" s="73">
+        <f>SUM(P5:P17)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="73">
+        <f>SUM(Q5:Q17)</f>
+        <v/>
+      </c>
+      <c r="R18" s="73">
+        <f>SUM(R5:R17)</f>
+        <v/>
+      </c>
+      <c r="S18" s="73">
+        <f>SUM(S5:S17)</f>
+        <v/>
+      </c>
+      <c r="T18" s="73">
+        <f>SUM(T5:T17)</f>
+        <v/>
+      </c>
+      <c r="U18" s="73">
+        <f>SUM(U5:U17)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:V2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A1:V1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A2:U2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Add per-person share of the take by role vs AUM
New 'Take per Person' sheet: one individual's share = role weight / total
weighted units, swept across AUM $100m -> $2bn. Every role's per-person
share declines monotonically as the firm hires. Adds native Excel line chart
and a line-chart PNG.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K14qB8MpeJ8Pk8H1GeEUV4
</commit_message>
<xml_diff>
--- a/Performance_Fee_Framework.xlsx
+++ b/Performance_Fee_Framework.xlsx
@@ -8,7 +8,8 @@
   <sheets>
     <sheet name="Static" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Take by AUM" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Take per Person" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -330,7 +331,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -494,6 +495,12 @@
     <xf numFmtId="3" fontId="25" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="23" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -573,7 +580,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -1075,6 +1081,510 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Per-person share of the take vs AUM</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$5:$U$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$6:$U$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A7</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$7:$U$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A8</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$8:$U$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$9:$U$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$10:$U$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$11:$U$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$12:$U$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A13</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$13:$U$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A14</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$14:$U$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A15</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$15:$U$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A16</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$16:$U$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
+          <tx>
+            <strRef>
+              <f>'Take per Person'!A17</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Take per Person'!$B$4:$U$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Take per Person'!$B$17:$U$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>AUM (USD m)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% of take per person</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0.0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -1102,6 +1612,33 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9360000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -5110,6 +5647,1067 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:U18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="18" max="18"/>
+    <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="7" customWidth="1" min="20" max="20"/>
+    <col width="7" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="61" t="inlineStr">
+        <is>
+          <t>Share of the take PER PERSON, by role, as AUM grows $100m → $2bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="62" t="inlineStr">
+        <is>
+          <t>Per-person share = role weight ÷ total weighted units. One individual's slice — declines for every role as the firm hires.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="72" t="inlineStr">
+        <is>
+          <t>AUM (USD m) →</t>
+        </is>
+      </c>
+      <c r="B4" s="74" t="n">
+        <v>100</v>
+      </c>
+      <c r="C4" s="74" t="n">
+        <v>200</v>
+      </c>
+      <c r="D4" s="74" t="n">
+        <v>300</v>
+      </c>
+      <c r="E4" s="74" t="n">
+        <v>400</v>
+      </c>
+      <c r="F4" s="74" t="n">
+        <v>500</v>
+      </c>
+      <c r="G4" s="74" t="n">
+        <v>600</v>
+      </c>
+      <c r="H4" s="74" t="n">
+        <v>700</v>
+      </c>
+      <c r="I4" s="74" t="n">
+        <v>800</v>
+      </c>
+      <c r="J4" s="74" t="n">
+        <v>900</v>
+      </c>
+      <c r="K4" s="74" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L4" s="74" t="n">
+        <v>1100</v>
+      </c>
+      <c r="M4" s="74" t="n">
+        <v>1200</v>
+      </c>
+      <c r="N4" s="74" t="n">
+        <v>1300</v>
+      </c>
+      <c r="O4" s="74" t="n">
+        <v>1400</v>
+      </c>
+      <c r="P4" s="74" t="n">
+        <v>1500</v>
+      </c>
+      <c r="Q4" s="74" t="n">
+        <v>1600</v>
+      </c>
+      <c r="R4" s="74" t="n">
+        <v>1700</v>
+      </c>
+      <c r="S4" s="74" t="n">
+        <v>1800</v>
+      </c>
+      <c r="T4" s="74" t="n">
+        <v>1900</v>
+      </c>
+      <c r="U4" s="74" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="68" t="inlineStr">
+        <is>
+          <t>Managing Partner / CIO  (wt 100)</t>
+        </is>
+      </c>
+      <c r="B5" s="75" t="n">
+        <v>0.4716981132075472</v>
+      </c>
+      <c r="C5" s="75" t="n">
+        <v>0.3745318352059925</v>
+      </c>
+      <c r="D5" s="75" t="n">
+        <v>0.3105590062111801</v>
+      </c>
+      <c r="E5" s="75" t="n">
+        <v>0.2604166666666667</v>
+      </c>
+      <c r="F5" s="75" t="n">
+        <v>0.2242152466367713</v>
+      </c>
+      <c r="G5" s="75" t="n">
+        <v>0.2152389151958674</v>
+      </c>
+      <c r="H5" s="75" t="n">
+        <v>0.206953642384106</v>
+      </c>
+      <c r="I5" s="75" t="n">
+        <v>0.1992825827022718</v>
+      </c>
+      <c r="J5" s="75" t="n">
+        <v>0.1921598770176787</v>
+      </c>
+      <c r="K5" s="75" t="n">
+        <v>0.1855287569573284</v>
+      </c>
+      <c r="L5" s="75" t="n">
+        <v>0.1803426510369703</v>
+      </c>
+      <c r="M5" s="75" t="n">
+        <v>0.1754385964912281</v>
+      </c>
+      <c r="N5" s="75" t="n">
+        <v>0.1707941929974381</v>
+      </c>
+      <c r="O5" s="75" t="n">
+        <v>0.1663893510815308</v>
+      </c>
+      <c r="P5" s="75" t="n">
+        <v>0.16220600162206</v>
+      </c>
+      <c r="Q5" s="75" t="n">
+        <v>0.1582278481012658</v>
+      </c>
+      <c r="R5" s="75" t="n">
+        <v>0.1544401544401544</v>
+      </c>
+      <c r="S5" s="75" t="n">
+        <v>0.1508295625942685</v>
+      </c>
+      <c r="T5" s="75" t="n">
+        <v>0.1473839351510685</v>
+      </c>
+      <c r="U5" s="75" t="n">
+        <v>0.1440922190201729</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="70" t="inlineStr">
+        <is>
+          <t>Partner / Co-PM  (wt 60)</t>
+        </is>
+      </c>
+      <c r="B6" s="76" t="n">
+        <v>0.2830188679245283</v>
+      </c>
+      <c r="C6" s="76" t="n">
+        <v>0.2247191011235955</v>
+      </c>
+      <c r="D6" s="76" t="n">
+        <v>0.1863354037267081</v>
+      </c>
+      <c r="E6" s="76" t="n">
+        <v>0.15625</v>
+      </c>
+      <c r="F6" s="76" t="n">
+        <v>0.1345291479820628</v>
+      </c>
+      <c r="G6" s="76" t="n">
+        <v>0.1291433491175205</v>
+      </c>
+      <c r="H6" s="76" t="n">
+        <v>0.1241721854304636</v>
+      </c>
+      <c r="I6" s="76" t="n">
+        <v>0.1195695496213631</v>
+      </c>
+      <c r="J6" s="76" t="n">
+        <v>0.1152959262106072</v>
+      </c>
+      <c r="K6" s="76" t="n">
+        <v>0.111317254174397</v>
+      </c>
+      <c r="L6" s="76" t="n">
+        <v>0.1082055906221821</v>
+      </c>
+      <c r="M6" s="76" t="n">
+        <v>0.1052631578947368</v>
+      </c>
+      <c r="N6" s="76" t="n">
+        <v>0.1024765157984629</v>
+      </c>
+      <c r="O6" s="76" t="n">
+        <v>0.09983361064891846</v>
+      </c>
+      <c r="P6" s="76" t="n">
+        <v>0.09732360097323602</v>
+      </c>
+      <c r="Q6" s="76" t="n">
+        <v>0.0949367088607595</v>
+      </c>
+      <c r="R6" s="76" t="n">
+        <v>0.09266409266409266</v>
+      </c>
+      <c r="S6" s="76" t="n">
+        <v>0.09049773755656108</v>
+      </c>
+      <c r="T6" s="76" t="n">
+        <v>0.08843036109064112</v>
+      </c>
+      <c r="U6" s="76" t="n">
+        <v>0.08645533141210375</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="68" t="inlineStr">
+        <is>
+          <t>Portfolio Manager  (wt 40)</t>
+        </is>
+      </c>
+      <c r="B7" s="75" t="n">
+        <v>0.1886792452830189</v>
+      </c>
+      <c r="C7" s="75" t="n">
+        <v>0.149812734082397</v>
+      </c>
+      <c r="D7" s="75" t="n">
+        <v>0.124223602484472</v>
+      </c>
+      <c r="E7" s="75" t="n">
+        <v>0.1041666666666667</v>
+      </c>
+      <c r="F7" s="75" t="n">
+        <v>0.08968609865470852</v>
+      </c>
+      <c r="G7" s="75" t="n">
+        <v>0.08609556607834697</v>
+      </c>
+      <c r="H7" s="75" t="n">
+        <v>0.08278145695364239</v>
+      </c>
+      <c r="I7" s="75" t="n">
+        <v>0.07971303308090873</v>
+      </c>
+      <c r="J7" s="75" t="n">
+        <v>0.07686395080707147</v>
+      </c>
+      <c r="K7" s="75" t="n">
+        <v>0.07421150278293136</v>
+      </c>
+      <c r="L7" s="75" t="n">
+        <v>0.0721370604147881</v>
+      </c>
+      <c r="M7" s="75" t="n">
+        <v>0.07017543859649122</v>
+      </c>
+      <c r="N7" s="75" t="n">
+        <v>0.06831767719897523</v>
+      </c>
+      <c r="O7" s="75" t="n">
+        <v>0.06655574043261231</v>
+      </c>
+      <c r="P7" s="75" t="n">
+        <v>0.064882400648824</v>
+      </c>
+      <c r="Q7" s="75" t="n">
+        <v>0.06329113924050633</v>
+      </c>
+      <c r="R7" s="75" t="n">
+        <v>0.06177606177606178</v>
+      </c>
+      <c r="S7" s="75" t="n">
+        <v>0.06033182503770739</v>
+      </c>
+      <c r="T7" s="75" t="n">
+        <v>0.05895357406042741</v>
+      </c>
+      <c r="U7" s="75" t="n">
+        <v>0.05763688760806916</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="70" t="inlineStr">
+        <is>
+          <t>Head of Research  (wt 30)</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="n">
+        <v>0.1415094339622641</v>
+      </c>
+      <c r="C8" s="76" t="n">
+        <v>0.1123595505617977</v>
+      </c>
+      <c r="D8" s="76" t="n">
+        <v>0.09316770186335403</v>
+      </c>
+      <c r="E8" s="76" t="n">
+        <v>0.078125</v>
+      </c>
+      <c r="F8" s="76" t="n">
+        <v>0.06726457399103139</v>
+      </c>
+      <c r="G8" s="76" t="n">
+        <v>0.06457167455876023</v>
+      </c>
+      <c r="H8" s="76" t="n">
+        <v>0.06208609271523179</v>
+      </c>
+      <c r="I8" s="76" t="n">
+        <v>0.05978477481068155</v>
+      </c>
+      <c r="J8" s="76" t="n">
+        <v>0.0576479631053036</v>
+      </c>
+      <c r="K8" s="76" t="n">
+        <v>0.05565862708719851</v>
+      </c>
+      <c r="L8" s="76" t="n">
+        <v>0.05410279531109107</v>
+      </c>
+      <c r="M8" s="76" t="n">
+        <v>0.05263157894736842</v>
+      </c>
+      <c r="N8" s="76" t="n">
+        <v>0.05123825789923143</v>
+      </c>
+      <c r="O8" s="76" t="n">
+        <v>0.04991680532445923</v>
+      </c>
+      <c r="P8" s="76" t="n">
+        <v>0.04866180048661801</v>
+      </c>
+      <c r="Q8" s="76" t="n">
+        <v>0.04746835443037975</v>
+      </c>
+      <c r="R8" s="76" t="n">
+        <v>0.04633204633204633</v>
+      </c>
+      <c r="S8" s="76" t="n">
+        <v>0.04524886877828054</v>
+      </c>
+      <c r="T8" s="76" t="n">
+        <v>0.04421518054532056</v>
+      </c>
+      <c r="U8" s="76" t="n">
+        <v>0.04322766570605188</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="68" t="inlineStr">
+        <is>
+          <t>Senior Analyst  (wt 20)</t>
+        </is>
+      </c>
+      <c r="B9" s="75" t="n">
+        <v>0.09433962264150944</v>
+      </c>
+      <c r="C9" s="75" t="n">
+        <v>0.0749063670411985</v>
+      </c>
+      <c r="D9" s="75" t="n">
+        <v>0.06211180124223602</v>
+      </c>
+      <c r="E9" s="75" t="n">
+        <v>0.05208333333333334</v>
+      </c>
+      <c r="F9" s="75" t="n">
+        <v>0.04484304932735426</v>
+      </c>
+      <c r="G9" s="75" t="n">
+        <v>0.04304778303917348</v>
+      </c>
+      <c r="H9" s="75" t="n">
+        <v>0.0413907284768212</v>
+      </c>
+      <c r="I9" s="75" t="n">
+        <v>0.03985651654045436</v>
+      </c>
+      <c r="J9" s="75" t="n">
+        <v>0.03843197540353573</v>
+      </c>
+      <c r="K9" s="75" t="n">
+        <v>0.03710575139146568</v>
+      </c>
+      <c r="L9" s="75" t="n">
+        <v>0.03606853020739405</v>
+      </c>
+      <c r="M9" s="75" t="n">
+        <v>0.03508771929824561</v>
+      </c>
+      <c r="N9" s="75" t="n">
+        <v>0.03415883859948762</v>
+      </c>
+      <c r="O9" s="75" t="n">
+        <v>0.03327787021630615</v>
+      </c>
+      <c r="P9" s="75" t="n">
+        <v>0.032441200324412</v>
+      </c>
+      <c r="Q9" s="75" t="n">
+        <v>0.03164556962025317</v>
+      </c>
+      <c r="R9" s="75" t="n">
+        <v>0.03088803088803089</v>
+      </c>
+      <c r="S9" s="75" t="n">
+        <v>0.0301659125188537</v>
+      </c>
+      <c r="T9" s="75" t="n">
+        <v>0.02947678703021371</v>
+      </c>
+      <c r="U9" s="75" t="n">
+        <v>0.02881844380403458</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="70" t="inlineStr">
+        <is>
+          <t>Analyst  (wt 12)</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="n">
+        <v>0.05660377358490566</v>
+      </c>
+      <c r="C10" s="76" t="n">
+        <v>0.0449438202247191</v>
+      </c>
+      <c r="D10" s="76" t="n">
+        <v>0.03726708074534162</v>
+      </c>
+      <c r="E10" s="76" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="F10" s="76" t="n">
+        <v>0.02690582959641256</v>
+      </c>
+      <c r="G10" s="76" t="n">
+        <v>0.02582866982350409</v>
+      </c>
+      <c r="H10" s="76" t="n">
+        <v>0.02483443708609272</v>
+      </c>
+      <c r="I10" s="76" t="n">
+        <v>0.02391390992427262</v>
+      </c>
+      <c r="J10" s="76" t="n">
+        <v>0.02305918524212144</v>
+      </c>
+      <c r="K10" s="76" t="n">
+        <v>0.02226345083487941</v>
+      </c>
+      <c r="L10" s="76" t="n">
+        <v>0.02164111812443643</v>
+      </c>
+      <c r="M10" s="76" t="n">
+        <v>0.02105263157894737</v>
+      </c>
+      <c r="N10" s="76" t="n">
+        <v>0.02049530315969257</v>
+      </c>
+      <c r="O10" s="76" t="n">
+        <v>0.01996672212978369</v>
+      </c>
+      <c r="P10" s="76" t="n">
+        <v>0.0194647201946472</v>
+      </c>
+      <c r="Q10" s="76" t="n">
+        <v>0.0189873417721519</v>
+      </c>
+      <c r="R10" s="76" t="n">
+        <v>0.01853281853281853</v>
+      </c>
+      <c r="S10" s="76" t="n">
+        <v>0.01809954751131222</v>
+      </c>
+      <c r="T10" s="76" t="n">
+        <v>0.01768607221812822</v>
+      </c>
+      <c r="U10" s="76" t="n">
+        <v>0.01729106628242075</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="68" t="inlineStr">
+        <is>
+          <t>Junior Analyst  (wt 6)</t>
+        </is>
+      </c>
+      <c r="B11" s="75" t="n">
+        <v>0.02830188679245283</v>
+      </c>
+      <c r="C11" s="75" t="n">
+        <v>0.02247191011235955</v>
+      </c>
+      <c r="D11" s="75" t="n">
+        <v>0.01863354037267081</v>
+      </c>
+      <c r="E11" s="75" t="n">
+        <v>0.015625</v>
+      </c>
+      <c r="F11" s="75" t="n">
+        <v>0.01345291479820628</v>
+      </c>
+      <c r="G11" s="75" t="n">
+        <v>0.01291433491175204</v>
+      </c>
+      <c r="H11" s="75" t="n">
+        <v>0.01241721854304636</v>
+      </c>
+      <c r="I11" s="75" t="n">
+        <v>0.01195695496213631</v>
+      </c>
+      <c r="J11" s="75" t="n">
+        <v>0.01152959262106072</v>
+      </c>
+      <c r="K11" s="75" t="n">
+        <v>0.0111317254174397</v>
+      </c>
+      <c r="L11" s="75" t="n">
+        <v>0.01082055906221822</v>
+      </c>
+      <c r="M11" s="75" t="n">
+        <v>0.01052631578947368</v>
+      </c>
+      <c r="N11" s="75" t="n">
+        <v>0.01024765157984629</v>
+      </c>
+      <c r="O11" s="75" t="n">
+        <v>0.009983361064891847</v>
+      </c>
+      <c r="P11" s="75" t="n">
+        <v>0.009732360097323601</v>
+      </c>
+      <c r="Q11" s="75" t="n">
+        <v>0.00949367088607595</v>
+      </c>
+      <c r="R11" s="75" t="n">
+        <v>0.009266409266409266</v>
+      </c>
+      <c r="S11" s="75" t="n">
+        <v>0.009049773755656109</v>
+      </c>
+      <c r="T11" s="75" t="n">
+        <v>0.008843036109064112</v>
+      </c>
+      <c r="U11" s="75" t="n">
+        <v>0.008645533141210375</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="70" t="inlineStr">
+        <is>
+          <t>Head of Trading  (wt 18)</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="n">
+        <v>0.08490566037735849</v>
+      </c>
+      <c r="C12" s="76" t="n">
+        <v>0.06741573033707865</v>
+      </c>
+      <c r="D12" s="76" t="n">
+        <v>0.05590062111801242</v>
+      </c>
+      <c r="E12" s="76" t="n">
+        <v>0.046875</v>
+      </c>
+      <c r="F12" s="76" t="n">
+        <v>0.04035874439461883</v>
+      </c>
+      <c r="G12" s="76" t="n">
+        <v>0.03874300473525614</v>
+      </c>
+      <c r="H12" s="76" t="n">
+        <v>0.03725165562913908</v>
+      </c>
+      <c r="I12" s="76" t="n">
+        <v>0.03587086488640893</v>
+      </c>
+      <c r="J12" s="76" t="n">
+        <v>0.03458877786318216</v>
+      </c>
+      <c r="K12" s="76" t="n">
+        <v>0.03339517625231911</v>
+      </c>
+      <c r="L12" s="76" t="n">
+        <v>0.03246167718665464</v>
+      </c>
+      <c r="M12" s="76" t="n">
+        <v>0.03157894736842105</v>
+      </c>
+      <c r="N12" s="76" t="n">
+        <v>0.03074295473953886</v>
+      </c>
+      <c r="O12" s="76" t="n">
+        <v>0.02995008319467554</v>
+      </c>
+      <c r="P12" s="76" t="n">
+        <v>0.0291970802919708</v>
+      </c>
+      <c r="Q12" s="76" t="n">
+        <v>0.02848101265822785</v>
+      </c>
+      <c r="R12" s="76" t="n">
+        <v>0.0277992277992278</v>
+      </c>
+      <c r="S12" s="76" t="n">
+        <v>0.02714932126696833</v>
+      </c>
+      <c r="T12" s="76" t="n">
+        <v>0.02652910832719233</v>
+      </c>
+      <c r="U12" s="76" t="n">
+        <v>0.02593659942363112</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="68" t="inlineStr">
+        <is>
+          <t>Trader / Execution  (wt 10)</t>
+        </is>
+      </c>
+      <c r="B13" s="75" t="n">
+        <v>0.04716981132075472</v>
+      </c>
+      <c r="C13" s="75" t="n">
+        <v>0.03745318352059925</v>
+      </c>
+      <c r="D13" s="75" t="n">
+        <v>0.03105590062111801</v>
+      </c>
+      <c r="E13" s="75" t="n">
+        <v>0.02604166666666667</v>
+      </c>
+      <c r="F13" s="75" t="n">
+        <v>0.02242152466367713</v>
+      </c>
+      <c r="G13" s="75" t="n">
+        <v>0.02152389151958674</v>
+      </c>
+      <c r="H13" s="75" t="n">
+        <v>0.0206953642384106</v>
+      </c>
+      <c r="I13" s="75" t="n">
+        <v>0.01992825827022718</v>
+      </c>
+      <c r="J13" s="75" t="n">
+        <v>0.01921598770176787</v>
+      </c>
+      <c r="K13" s="75" t="n">
+        <v>0.01855287569573284</v>
+      </c>
+      <c r="L13" s="75" t="n">
+        <v>0.01803426510369702</v>
+      </c>
+      <c r="M13" s="75" t="n">
+        <v>0.01754385964912281</v>
+      </c>
+      <c r="N13" s="75" t="n">
+        <v>0.01707941929974381</v>
+      </c>
+      <c r="O13" s="75" t="n">
+        <v>0.01663893510815308</v>
+      </c>
+      <c r="P13" s="75" t="n">
+        <v>0.016220600162206</v>
+      </c>
+      <c r="Q13" s="75" t="n">
+        <v>0.01582278481012658</v>
+      </c>
+      <c r="R13" s="75" t="n">
+        <v>0.01544401544401544</v>
+      </c>
+      <c r="S13" s="75" t="n">
+        <v>0.01508295625942685</v>
+      </c>
+      <c r="T13" s="75" t="n">
+        <v>0.01473839351510685</v>
+      </c>
+      <c r="U13" s="75" t="n">
+        <v>0.01440922190201729</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="70" t="inlineStr">
+        <is>
+          <t>COO / Head of Operations  (wt 15)</t>
+        </is>
+      </c>
+      <c r="B14" s="76" t="n">
+        <v>0.07075471698113207</v>
+      </c>
+      <c r="C14" s="76" t="n">
+        <v>0.05617977528089887</v>
+      </c>
+      <c r="D14" s="76" t="n">
+        <v>0.04658385093167702</v>
+      </c>
+      <c r="E14" s="76" t="n">
+        <v>0.0390625</v>
+      </c>
+      <c r="F14" s="76" t="n">
+        <v>0.0336322869955157</v>
+      </c>
+      <c r="G14" s="76" t="n">
+        <v>0.03228583727938011</v>
+      </c>
+      <c r="H14" s="76" t="n">
+        <v>0.0310430463576159</v>
+      </c>
+      <c r="I14" s="76" t="n">
+        <v>0.02989238740534077</v>
+      </c>
+      <c r="J14" s="76" t="n">
+        <v>0.0288239815526518</v>
+      </c>
+      <c r="K14" s="76" t="n">
+        <v>0.02782931354359926</v>
+      </c>
+      <c r="L14" s="76" t="n">
+        <v>0.02705139765554554</v>
+      </c>
+      <c r="M14" s="76" t="n">
+        <v>0.02631578947368421</v>
+      </c>
+      <c r="N14" s="76" t="n">
+        <v>0.02561912894961571</v>
+      </c>
+      <c r="O14" s="76" t="n">
+        <v>0.02495840266222962</v>
+      </c>
+      <c r="P14" s="76" t="n">
+        <v>0.024330900243309</v>
+      </c>
+      <c r="Q14" s="76" t="n">
+        <v>0.02373417721518987</v>
+      </c>
+      <c r="R14" s="76" t="n">
+        <v>0.02316602316602316</v>
+      </c>
+      <c r="S14" s="76" t="n">
+        <v>0.02262443438914027</v>
+      </c>
+      <c r="T14" s="76" t="n">
+        <v>0.02210759027266028</v>
+      </c>
+      <c r="U14" s="76" t="n">
+        <v>0.02161383285302594</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="68" t="inlineStr">
+        <is>
+          <t>CFO / Finance  (wt 12)</t>
+        </is>
+      </c>
+      <c r="B15" s="75" t="n">
+        <v>0.05660377358490566</v>
+      </c>
+      <c r="C15" s="75" t="n">
+        <v>0.0449438202247191</v>
+      </c>
+      <c r="D15" s="75" t="n">
+        <v>0.03726708074534162</v>
+      </c>
+      <c r="E15" s="75" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="F15" s="75" t="n">
+        <v>0.02690582959641256</v>
+      </c>
+      <c r="G15" s="75" t="n">
+        <v>0.02582866982350409</v>
+      </c>
+      <c r="H15" s="75" t="n">
+        <v>0.02483443708609272</v>
+      </c>
+      <c r="I15" s="75" t="n">
+        <v>0.02391390992427262</v>
+      </c>
+      <c r="J15" s="75" t="n">
+        <v>0.02305918524212144</v>
+      </c>
+      <c r="K15" s="75" t="n">
+        <v>0.02226345083487941</v>
+      </c>
+      <c r="L15" s="75" t="n">
+        <v>0.02164111812443643</v>
+      </c>
+      <c r="M15" s="75" t="n">
+        <v>0.02105263157894737</v>
+      </c>
+      <c r="N15" s="75" t="n">
+        <v>0.02049530315969257</v>
+      </c>
+      <c r="O15" s="75" t="n">
+        <v>0.01996672212978369</v>
+      </c>
+      <c r="P15" s="75" t="n">
+        <v>0.0194647201946472</v>
+      </c>
+      <c r="Q15" s="75" t="n">
+        <v>0.0189873417721519</v>
+      </c>
+      <c r="R15" s="75" t="n">
+        <v>0.01853281853281853</v>
+      </c>
+      <c r="S15" s="75" t="n">
+        <v>0.01809954751131222</v>
+      </c>
+      <c r="T15" s="75" t="n">
+        <v>0.01768607221812822</v>
+      </c>
+      <c r="U15" s="75" t="n">
+        <v>0.01729106628242075</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="70" t="inlineStr">
+        <is>
+          <t>Compliance / Legal  (wt 8)</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="n">
+        <v>0.03773584905660377</v>
+      </c>
+      <c r="C16" s="76" t="n">
+        <v>0.0299625468164794</v>
+      </c>
+      <c r="D16" s="76" t="n">
+        <v>0.02484472049689441</v>
+      </c>
+      <c r="E16" s="76" t="n">
+        <v>0.02083333333333333</v>
+      </c>
+      <c r="F16" s="76" t="n">
+        <v>0.0179372197309417</v>
+      </c>
+      <c r="G16" s="76" t="n">
+        <v>0.01721911321566939</v>
+      </c>
+      <c r="H16" s="76" t="n">
+        <v>0.01655629139072848</v>
+      </c>
+      <c r="I16" s="76" t="n">
+        <v>0.01594260661618175</v>
+      </c>
+      <c r="J16" s="76" t="n">
+        <v>0.01537279016141429</v>
+      </c>
+      <c r="K16" s="76" t="n">
+        <v>0.01484230055658627</v>
+      </c>
+      <c r="L16" s="76" t="n">
+        <v>0.01442741208295762</v>
+      </c>
+      <c r="M16" s="76" t="n">
+        <v>0.01403508771929825</v>
+      </c>
+      <c r="N16" s="76" t="n">
+        <v>0.01366353543979505</v>
+      </c>
+      <c r="O16" s="76" t="n">
+        <v>0.01331114808652246</v>
+      </c>
+      <c r="P16" s="76" t="n">
+        <v>0.0129764801297648</v>
+      </c>
+      <c r="Q16" s="76" t="n">
+        <v>0.01265822784810127</v>
+      </c>
+      <c r="R16" s="76" t="n">
+        <v>0.01235521235521236</v>
+      </c>
+      <c r="S16" s="76" t="n">
+        <v>0.01206636500754148</v>
+      </c>
+      <c r="T16" s="76" t="n">
+        <v>0.01179071481208548</v>
+      </c>
+      <c r="U16" s="76" t="n">
+        <v>0.01152737752161383</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="68" t="inlineStr">
+        <is>
+          <t>Investor Relations / Ops  (wt 5)</t>
+        </is>
+      </c>
+      <c r="B17" s="75" t="n">
+        <v>0.02358490566037736</v>
+      </c>
+      <c r="C17" s="75" t="n">
+        <v>0.01872659176029963</v>
+      </c>
+      <c r="D17" s="75" t="n">
+        <v>0.01552795031055901</v>
+      </c>
+      <c r="E17" s="75" t="n">
+        <v>0.01302083333333333</v>
+      </c>
+      <c r="F17" s="75" t="n">
+        <v>0.01121076233183856</v>
+      </c>
+      <c r="G17" s="75" t="n">
+        <v>0.01076194575979337</v>
+      </c>
+      <c r="H17" s="75" t="n">
+        <v>0.0103476821192053</v>
+      </c>
+      <c r="I17" s="75" t="n">
+        <v>0.009964129135113591</v>
+      </c>
+      <c r="J17" s="75" t="n">
+        <v>0.009607993850883933</v>
+      </c>
+      <c r="K17" s="75" t="n">
+        <v>0.00927643784786642</v>
+      </c>
+      <c r="L17" s="75" t="n">
+        <v>0.009017132551848512</v>
+      </c>
+      <c r="M17" s="75" t="n">
+        <v>0.008771929824561403</v>
+      </c>
+      <c r="N17" s="75" t="n">
+        <v>0.008539709649871904</v>
+      </c>
+      <c r="O17" s="75" t="n">
+        <v>0.008319467554076539</v>
+      </c>
+      <c r="P17" s="75" t="n">
+        <v>0.008110300081103</v>
+      </c>
+      <c r="Q17" s="75" t="n">
+        <v>0.007911392405063292</v>
+      </c>
+      <c r="R17" s="75" t="n">
+        <v>0.007722007722007722</v>
+      </c>
+      <c r="S17" s="75" t="n">
+        <v>0.007541478129713424</v>
+      </c>
+      <c r="T17" s="75" t="n">
+        <v>0.007369196757553427</v>
+      </c>
+      <c r="U17" s="75" t="n">
+        <v>0.007204610951008645</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="72" t="inlineStr">
+        <is>
+          <t>Total units (denominator)</t>
+        </is>
+      </c>
+      <c r="B18" s="74" t="n">
+        <v>212</v>
+      </c>
+      <c r="C18" s="74" t="n">
+        <v>267</v>
+      </c>
+      <c r="D18" s="74" t="n">
+        <v>322</v>
+      </c>
+      <c r="E18" s="74" t="n">
+        <v>384</v>
+      </c>
+      <c r="F18" s="74" t="n">
+        <v>446</v>
+      </c>
+      <c r="G18" s="74" t="n">
+        <v>465</v>
+      </c>
+      <c r="H18" s="74" t="n">
+        <v>483</v>
+      </c>
+      <c r="I18" s="74" t="n">
+        <v>502</v>
+      </c>
+      <c r="J18" s="74" t="n">
+        <v>520</v>
+      </c>
+      <c r="K18" s="74" t="n">
+        <v>539</v>
+      </c>
+      <c r="L18" s="74" t="n">
+        <v>554</v>
+      </c>
+      <c r="M18" s="74" t="n">
+        <v>570</v>
+      </c>
+      <c r="N18" s="74" t="n">
+        <v>586</v>
+      </c>
+      <c r="O18" s="74" t="n">
+        <v>601</v>
+      </c>
+      <c r="P18" s="74" t="n">
+        <v>616</v>
+      </c>
+      <c r="Q18" s="74" t="n">
+        <v>632</v>
+      </c>
+      <c r="R18" s="74" t="n">
+        <v>648</v>
+      </c>
+      <c r="S18" s="74" t="n">
+        <v>663</v>
+      </c>
+      <c r="T18" s="74" t="n">
+        <v>678</v>
+      </c>
+      <c r="U18" s="74" t="n">
+        <v>694</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A2:U2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:V34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>

</xml_diff>

<commit_message>
Add profit simulation by AUM level with ownership distribution
New 'Profit Simulation' sheet: firm EBIT = management fee (1.5% x AUM) +
equity take (40% of performance fee) - operating costs (loaded salaries +
other costs), at each AUM scenario. EBIT distributed by ownership: CIO 63.6%,
two PMs 10% each, other 16.4%. EBIT at $20m reconciles exactly with source
sheet (-1.4174). Links to Static; ownership % and other-cost cells editable.
Adds native Excel bar/line charts and a two-panel PNG.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K14qB8MpeJ8Pk8H1GeEUV4
</commit_message>
<xml_diff>
--- a/Performance_Fee_Framework.xlsx
+++ b/Performance_Fee_Framework.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Static" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Take by AUM" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Take per Person" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Profit Simulation" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -80,7 +81,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -122,8 +123,13 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -145,11 +151,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -269,6 +319,59 @@
     <xf numFmtId="165" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -347,7 +450,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -851,7 +953,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -1353,6 +1454,287 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Firm EBIT by AUM level (millions)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Profit Simulation'!A14</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Profit Simulation'!$H$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Profit Simulation'!$B$14:$G$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Profit to each owner (millions)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Profit Simulation'!A18</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Profit Simulation'!$H$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Profit Simulation'!$B$18:$G$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Profit Simulation'!A19</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Profit Simulation'!$H$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Profit Simulation'!$B$19:$G$19</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Profit Simulation'!A20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Profit Simulation'!$H$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Profit Simulation'!$B$20:$G$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Profit Simulation'!A21</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Profit Simulation'!$H$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Profit Simulation'!$B$21:$G$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>millions</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -1399,6 +1781,55 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1741,6 +2172,10 @@
           <t>Performance-fee rate (of profits)</t>
         </is>
       </c>
+      <c r="B5" s="45" t="n"/>
+      <c r="C5" s="45" t="n"/>
+      <c r="D5" s="45" t="n"/>
+      <c r="E5" s="46" t="n"/>
       <c r="F5" s="5" t="n">
         <v>0.2</v>
       </c>
@@ -1751,6 +2186,10 @@
           <t>Firm take rate — share of perf-fee to the comp pool</t>
         </is>
       </c>
+      <c r="B6" s="45" t="n"/>
+      <c r="C6" s="45" t="n"/>
+      <c r="D6" s="45" t="n"/>
+      <c r="E6" s="46" t="n"/>
       <c r="F6" s="5" t="n">
         <v>0.6</v>
       </c>
@@ -1761,6 +2200,10 @@
           <t>Assumed gross return on AUM</t>
         </is>
       </c>
+      <c r="B7" s="45" t="n"/>
+      <c r="C7" s="45" t="n"/>
+      <c r="D7" s="45" t="n"/>
+      <c r="E7" s="46" t="n"/>
       <c r="F7" s="5" t="n">
         <v>0.12</v>
       </c>
@@ -1771,6 +2214,10 @@
           <t>Management fee (of AUM)</t>
         </is>
       </c>
+      <c r="B8" s="45" t="n"/>
+      <c r="C8" s="45" t="n"/>
+      <c r="D8" s="45" t="n"/>
+      <c r="E8" s="46" t="n"/>
       <c r="F8" s="5" t="n">
         <v>0.015</v>
       </c>
@@ -1781,6 +2228,10 @@
           <t>AUM tier threshold (millions)</t>
         </is>
       </c>
+      <c r="B9" s="45" t="n"/>
+      <c r="C9" s="45" t="n"/>
+      <c r="D9" s="45" t="n"/>
+      <c r="E9" s="46" t="n"/>
       <c r="F9" s="6" t="n">
         <v>300</v>
       </c>
@@ -1791,6 +2242,10 @@
           <t>Employer cost loading on salary</t>
         </is>
       </c>
+      <c r="B10" s="45" t="n"/>
+      <c r="C10" s="45" t="n"/>
+      <c r="D10" s="45" t="n"/>
+      <c r="E10" s="46" t="n"/>
       <c r="F10" s="7" t="n">
         <v>1.62</v>
       </c>
@@ -6291,4 +6746,608 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>Profit simulation by AUM level, with ownership distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="48" t="inlineStr">
+        <is>
+          <t>Firm EBIT = management fee + equity take (40% of perf fee) − operating costs. Distributed to owners. Millions; links to Static.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>P&amp;L line  (millions)</t>
+        </is>
+      </c>
+      <c r="H4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $20m</t>
+        </is>
+      </c>
+      <c r="I4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $300m</t>
+        </is>
+      </c>
+      <c r="J4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $500m</t>
+        </is>
+      </c>
+      <c r="K4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $1,000m</t>
+        </is>
+      </c>
+      <c r="L4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $2,000m</t>
+        </is>
+      </c>
+      <c r="M4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $5,000m</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>AUM</t>
+        </is>
+      </c>
+      <c r="H5" s="50">
+        <f>Static!H15</f>
+        <v/>
+      </c>
+      <c r="I5" s="50">
+        <f>Static!I15</f>
+        <v/>
+      </c>
+      <c r="J5" s="50">
+        <f>Static!J15</f>
+        <v/>
+      </c>
+      <c r="K5" s="50">
+        <f>Static!K15</f>
+        <v/>
+      </c>
+      <c r="L5" s="50">
+        <f>Static!L15</f>
+        <v/>
+      </c>
+      <c r="M5" s="50">
+        <f>Static!M15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Management fee  (1.5% × AUM)</t>
+        </is>
+      </c>
+      <c r="H6" s="51">
+        <f>Static!H15*Static!$F$8</f>
+        <v/>
+      </c>
+      <c r="I6" s="51">
+        <f>Static!I15*Static!$F$8</f>
+        <v/>
+      </c>
+      <c r="J6" s="51">
+        <f>Static!J15*Static!$F$8</f>
+        <v/>
+      </c>
+      <c r="K6" s="51">
+        <f>Static!K15*Static!$F$8</f>
+        <v/>
+      </c>
+      <c r="L6" s="51">
+        <f>Static!L15*Static!$F$8</f>
+        <v/>
+      </c>
+      <c r="M6" s="51">
+        <f>Static!M15*Static!$F$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Performance fee  (20% × profit)</t>
+        </is>
+      </c>
+      <c r="H7" s="51">
+        <f>Static!H15*Static!$F$7*Static!$F$5</f>
+        <v/>
+      </c>
+      <c r="I7" s="51">
+        <f>Static!I15*Static!$F$7*Static!$F$5</f>
+        <v/>
+      </c>
+      <c r="J7" s="51">
+        <f>Static!J15*Static!$F$7*Static!$F$5</f>
+        <v/>
+      </c>
+      <c r="K7" s="51">
+        <f>Static!K15*Static!$F$7*Static!$F$5</f>
+        <v/>
+      </c>
+      <c r="L7" s="51">
+        <f>Static!L15*Static!$F$7*Static!$F$5</f>
+        <v/>
+      </c>
+      <c r="M7" s="51">
+        <f>Static!M15*Static!$F$7*Static!$F$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which team take (60%) → staff</t>
+        </is>
+      </c>
+      <c r="H8" s="53">
+        <f>H7*Static!$F$6</f>
+        <v/>
+      </c>
+      <c r="I8" s="53">
+        <f>I7*Static!$F$6</f>
+        <v/>
+      </c>
+      <c r="J8" s="53">
+        <f>J7*Static!$F$6</f>
+        <v/>
+      </c>
+      <c r="K8" s="53">
+        <f>K7*Static!$F$6</f>
+        <v/>
+      </c>
+      <c r="L8" s="53">
+        <f>L7*Static!$F$6</f>
+        <v/>
+      </c>
+      <c r="M8" s="53">
+        <f>M7*Static!$F$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which equity take (40%) → firm</t>
+        </is>
+      </c>
+      <c r="H9" s="51">
+        <f>H7*(1-Static!$F$6)</f>
+        <v/>
+      </c>
+      <c r="I9" s="51">
+        <f>I7*(1-Static!$F$6)</f>
+        <v/>
+      </c>
+      <c r="J9" s="51">
+        <f>J7*(1-Static!$F$6)</f>
+        <v/>
+      </c>
+      <c r="K9" s="51">
+        <f>K7*(1-Static!$F$6)</f>
+        <v/>
+      </c>
+      <c r="L9" s="51">
+        <f>L7*(1-Static!$F$6)</f>
+        <v/>
+      </c>
+      <c r="M9" s="51">
+        <f>M7*(1-Static!$F$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Firm revenue  (mgmt fee + equity take)</t>
+        </is>
+      </c>
+      <c r="H10" s="54">
+        <f>H6+H9</f>
+        <v/>
+      </c>
+      <c r="I10" s="54">
+        <f>I6+I9</f>
+        <v/>
+      </c>
+      <c r="J10" s="54">
+        <f>J6+J9</f>
+        <v/>
+      </c>
+      <c r="K10" s="54">
+        <f>K6+K9</f>
+        <v/>
+      </c>
+      <c r="L10" s="54">
+        <f>L6+L9</f>
+        <v/>
+      </c>
+      <c r="M10" s="54">
+        <f>M6+M9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Operating cost: loaded salaries</t>
+        </is>
+      </c>
+      <c r="H11" s="51">
+        <f>Static!H36</f>
+        <v/>
+      </c>
+      <c r="I11" s="51">
+        <f>Static!I36</f>
+        <v/>
+      </c>
+      <c r="J11" s="51">
+        <f>Static!J36</f>
+        <v/>
+      </c>
+      <c r="K11" s="51">
+        <f>Static!K36</f>
+        <v/>
+      </c>
+      <c r="L11" s="51">
+        <f>Static!L36</f>
+        <v/>
+      </c>
+      <c r="M11" s="51">
+        <f>Static!M36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="55" t="inlineStr">
+        <is>
+          <t>Operating cost: other costs</t>
+        </is>
+      </c>
+      <c r="H12" s="56" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I12" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="56" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K12" s="56" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" s="56" t="n">
+        <v>4.301</v>
+      </c>
+      <c r="M12" s="56" t="n">
+        <v>4.301</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="57" t="inlineStr">
+        <is>
+          <t>Total operating costs</t>
+        </is>
+      </c>
+      <c r="H13" s="58">
+        <f>H11+H12</f>
+        <v/>
+      </c>
+      <c r="I13" s="58">
+        <f>I11+I12</f>
+        <v/>
+      </c>
+      <c r="J13" s="58">
+        <f>J11+J12</f>
+        <v/>
+      </c>
+      <c r="K13" s="58">
+        <f>K11+K12</f>
+        <v/>
+      </c>
+      <c r="L13" s="58">
+        <f>L11+L12</f>
+        <v/>
+      </c>
+      <c r="M13" s="58">
+        <f>M11+M12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>EBIT  (profit to owners)</t>
+        </is>
+      </c>
+      <c r="H14" s="59">
+        <f>H10-H13</f>
+        <v/>
+      </c>
+      <c r="I14" s="59">
+        <f>I10-I13</f>
+        <v/>
+      </c>
+      <c r="J14" s="59">
+        <f>J10-J13</f>
+        <v/>
+      </c>
+      <c r="K14" s="59">
+        <f>K10-K13</f>
+        <v/>
+      </c>
+      <c r="L14" s="59">
+        <f>L10-L13</f>
+        <v/>
+      </c>
+      <c r="M14" s="59">
+        <f>M10-M13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="52" t="inlineStr">
+        <is>
+          <t>EBIT margin (on firm revenue)</t>
+        </is>
+      </c>
+      <c r="H15" s="60">
+        <f>IF(H10=0,0,H14/H10)</f>
+        <v/>
+      </c>
+      <c r="I15" s="60">
+        <f>IF(I10=0,0,I14/I10)</f>
+        <v/>
+      </c>
+      <c r="J15" s="60">
+        <f>IF(J10=0,0,J14/J10)</f>
+        <v/>
+      </c>
+      <c r="K15" s="60">
+        <f>IF(K10=0,0,K14/K10)</f>
+        <v/>
+      </c>
+      <c r="L15" s="60">
+        <f>IF(L10=0,0,L14/L10)</f>
+        <v/>
+      </c>
+      <c r="M15" s="60">
+        <f>IF(M10=0,0,M14/M10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Ownership distribution of EBIT</t>
+        </is>
+      </c>
+      <c r="H17" s="49" t="inlineStr"/>
+      <c r="I17" s="49" t="inlineStr"/>
+      <c r="J17" s="49" t="inlineStr"/>
+      <c r="K17" s="49" t="inlineStr"/>
+      <c r="L17" s="49" t="inlineStr"/>
+      <c r="M17" s="49" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>CIO</t>
+        </is>
+      </c>
+      <c r="G18" s="61" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="H18" s="62">
+        <f>H14*$G18</f>
+        <v/>
+      </c>
+      <c r="I18" s="62">
+        <f>I14*$G18</f>
+        <v/>
+      </c>
+      <c r="J18" s="62">
+        <f>J14*$G18</f>
+        <v/>
+      </c>
+      <c r="K18" s="62">
+        <f>K14*$G18</f>
+        <v/>
+      </c>
+      <c r="L18" s="62">
+        <f>L14*$G18</f>
+        <v/>
+      </c>
+      <c r="M18" s="62">
+        <f>M14*$G18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Portfolio Manager 1</t>
+        </is>
+      </c>
+      <c r="G19" s="61" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H19" s="51">
+        <f>H14*$G19</f>
+        <v/>
+      </c>
+      <c r="I19" s="51">
+        <f>I14*$G19</f>
+        <v/>
+      </c>
+      <c r="J19" s="51">
+        <f>J14*$G19</f>
+        <v/>
+      </c>
+      <c r="K19" s="51">
+        <f>K14*$G19</f>
+        <v/>
+      </c>
+      <c r="L19" s="51">
+        <f>L14*$G19</f>
+        <v/>
+      </c>
+      <c r="M19" s="51">
+        <f>M14*$G19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Portfolio Manager 2</t>
+        </is>
+      </c>
+      <c r="G20" s="61" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H20" s="62">
+        <f>H14*$G20</f>
+        <v/>
+      </c>
+      <c r="I20" s="62">
+        <f>I14*$G20</f>
+        <v/>
+      </c>
+      <c r="J20" s="62">
+        <f>J14*$G20</f>
+        <v/>
+      </c>
+      <c r="K20" s="62">
+        <f>K14*$G20</f>
+        <v/>
+      </c>
+      <c r="L20" s="62">
+        <f>L14*$G20</f>
+        <v/>
+      </c>
+      <c r="M20" s="62">
+        <f>M14*$G20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Other owners</t>
+        </is>
+      </c>
+      <c r="G21" s="61" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="H21" s="51">
+        <f>H14*$G21</f>
+        <v/>
+      </c>
+      <c r="I21" s="51">
+        <f>I14*$G21</f>
+        <v/>
+      </c>
+      <c r="J21" s="51">
+        <f>J14*$G21</f>
+        <v/>
+      </c>
+      <c r="K21" s="51">
+        <f>K14*$G21</f>
+        <v/>
+      </c>
+      <c r="L21" s="51">
+        <f>L14*$G21</f>
+        <v/>
+      </c>
+      <c r="M21" s="51">
+        <f>M14*$G21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>Total distributed</t>
+        </is>
+      </c>
+      <c r="G22" s="63">
+        <f>SUM(G18:G21)</f>
+        <v/>
+      </c>
+      <c r="H22" s="54">
+        <f>SUM(H18:H21)</f>
+        <v/>
+      </c>
+      <c r="I22" s="54">
+        <f>SUM(I18:I21)</f>
+        <v/>
+      </c>
+      <c r="J22" s="54">
+        <f>SUM(J18:J21)</f>
+        <v/>
+      </c>
+      <c r="K22" s="54">
+        <f>SUM(K18:K21)</f>
+        <v/>
+      </c>
+      <c r="L22" s="54">
+        <f>SUM(L18:L21)</f>
+        <v/>
+      </c>
+      <c r="M22" s="54">
+        <f>SUM(M18:M21)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add overall comp for equity owners (CIO + two PMs)
New 'Owner Total Comp' sheet: total comp = base salary + performance take
(weight x unit value) + equity distribution (ownership% x EBIT), per AUM
level, for CIO (equity 63.6%) and the two PMs (10% each). Formulas link to
Static (salary, weight, unit value) and Profit Simulation (EBIT). Adds native
Excel bar chart and a 3-panel stacked PNG showing the salary/performance/
equity composition.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K14qB8MpeJ8Pk8H1GeEUV4
</commit_message>
<xml_diff>
--- a/Performance_Fee_Framework.xlsx
+++ b/Performance_Fee_Framework.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Take by AUM" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Take per Person" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Profit Simulation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Owner Total Comp" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.000"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,6 +80,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="10">
@@ -199,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -370,6 +376,19 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1735,6 +1754,112 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Total comp: CIO vs PM (each), by AUM (millions)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Owner Total Comp'!A9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Owner Total Comp'!$H$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Owner Total Comp'!$B$9:$G$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Owner Total Comp'!A14</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Owner Total Comp'!$H$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Owner Total Comp'!$B$14:$G$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -1830,6 +1955,33 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -7350,4 +7502,540 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>Total compensation for equity owners — CIO and the two PMs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="48" t="inlineStr">
+        <is>
+          <t>Total comp = base salary + performance take (weight × unit value) + equity distribution (ownership × EBIT). Millions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Component  (millions)</t>
+        </is>
+      </c>
+      <c r="H4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $20m</t>
+        </is>
+      </c>
+      <c r="I4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $300m</t>
+        </is>
+      </c>
+      <c r="J4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $500m</t>
+        </is>
+      </c>
+      <c r="K4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $1,000m</t>
+        </is>
+      </c>
+      <c r="L4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $2,000m</t>
+        </is>
+      </c>
+      <c r="M4" s="49" t="inlineStr">
+        <is>
+          <t>AUM $5,000m</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="64" t="inlineStr">
+        <is>
+          <t>CIO  (wt 16, equity 63.6%)</t>
+        </is>
+      </c>
+      <c r="H5" s="65" t="inlineStr"/>
+      <c r="I5" s="65" t="inlineStr"/>
+      <c r="J5" s="65" t="inlineStr"/>
+      <c r="K5" s="65" t="inlineStr"/>
+      <c r="L5" s="65" t="inlineStr"/>
+      <c r="M5" s="65" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Base salary</t>
+        </is>
+      </c>
+      <c r="H6" s="51">
+        <f>IF(Static!H15&lt;Static!$F$9,Static!$B$21,Static!$C$21)</f>
+        <v/>
+      </c>
+      <c r="I6" s="51">
+        <f>IF(Static!I15&lt;Static!$F$9,Static!$B$21,Static!$C$21)</f>
+        <v/>
+      </c>
+      <c r="J6" s="51">
+        <f>IF(Static!J15&lt;Static!$F$9,Static!$B$21,Static!$C$21)</f>
+        <v/>
+      </c>
+      <c r="K6" s="51">
+        <f>IF(Static!K15&lt;Static!$F$9,Static!$B$21,Static!$C$21)</f>
+        <v/>
+      </c>
+      <c r="L6" s="51">
+        <f>IF(Static!L15&lt;Static!$F$9,Static!$B$21,Static!$C$21)</f>
+        <v/>
+      </c>
+      <c r="M6" s="51">
+        <f>IF(Static!M15&lt;Static!$F$9,Static!$B$21,Static!$C$21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Performance take  (weight × unit value)</t>
+        </is>
+      </c>
+      <c r="H7" s="51">
+        <f>Static!$D$21*Static!H$35</f>
+        <v/>
+      </c>
+      <c r="I7" s="51">
+        <f>Static!$D$21*Static!I$35</f>
+        <v/>
+      </c>
+      <c r="J7" s="51">
+        <f>Static!$D$21*Static!J$35</f>
+        <v/>
+      </c>
+      <c r="K7" s="51">
+        <f>Static!$D$21*Static!K$35</f>
+        <v/>
+      </c>
+      <c r="L7" s="51">
+        <f>Static!$D$21*Static!L$35</f>
+        <v/>
+      </c>
+      <c r="M7" s="51">
+        <f>Static!$D$21*Static!M$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Equity distribution  (63.6% × EBIT)</t>
+        </is>
+      </c>
+      <c r="G8" s="61" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="H8" s="66">
+        <f>'Profit Simulation'!H14*$G8</f>
+        <v/>
+      </c>
+      <c r="I8" s="66">
+        <f>'Profit Simulation'!I14*$G8</f>
+        <v/>
+      </c>
+      <c r="J8" s="66">
+        <f>'Profit Simulation'!J14*$G8</f>
+        <v/>
+      </c>
+      <c r="K8" s="66">
+        <f>'Profit Simulation'!K14*$G8</f>
+        <v/>
+      </c>
+      <c r="L8" s="66">
+        <f>'Profit Simulation'!L14*$G8</f>
+        <v/>
+      </c>
+      <c r="M8" s="66">
+        <f>'Profit Simulation'!M14*$G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TOTAL COMP — CIO</t>
+        </is>
+      </c>
+      <c r="H9" s="54">
+        <f>SUM(H6:H8)</f>
+        <v/>
+      </c>
+      <c r="I9" s="54">
+        <f>SUM(I6:I8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="54">
+        <f>SUM(J6:J8)</f>
+        <v/>
+      </c>
+      <c r="K9" s="54">
+        <f>SUM(K6:K8)</f>
+        <v/>
+      </c>
+      <c r="L9" s="54">
+        <f>SUM(L6:L8)</f>
+        <v/>
+      </c>
+      <c r="M9" s="54">
+        <f>SUM(M6:M8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="64" t="inlineStr">
+        <is>
+          <t>Portfolio Manager 1  (wt 8, equity 10.0%)</t>
+        </is>
+      </c>
+      <c r="H11" s="65" t="inlineStr"/>
+      <c r="I11" s="65" t="inlineStr"/>
+      <c r="J11" s="65" t="inlineStr"/>
+      <c r="K11" s="65" t="inlineStr"/>
+      <c r="L11" s="65" t="inlineStr"/>
+      <c r="M11" s="65" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Base salary</t>
+        </is>
+      </c>
+      <c r="H12" s="51">
+        <f>IF(Static!H15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+      <c r="I12" s="51">
+        <f>IF(Static!I15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+      <c r="J12" s="51">
+        <f>IF(Static!J15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+      <c r="K12" s="51">
+        <f>IF(Static!K15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+      <c r="L12" s="51">
+        <f>IF(Static!L15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+      <c r="M12" s="51">
+        <f>IF(Static!M15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Performance take  (weight × unit value)</t>
+        </is>
+      </c>
+      <c r="H13" s="51">
+        <f>Static!$D$22*Static!H$35</f>
+        <v/>
+      </c>
+      <c r="I13" s="51">
+        <f>Static!$D$22*Static!I$35</f>
+        <v/>
+      </c>
+      <c r="J13" s="51">
+        <f>Static!$D$22*Static!J$35</f>
+        <v/>
+      </c>
+      <c r="K13" s="51">
+        <f>Static!$D$22*Static!K$35</f>
+        <v/>
+      </c>
+      <c r="L13" s="51">
+        <f>Static!$D$22*Static!L$35</f>
+        <v/>
+      </c>
+      <c r="M13" s="51">
+        <f>Static!$D$22*Static!M$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Equity distribution  (10.0% × EBIT)</t>
+        </is>
+      </c>
+      <c r="G14" s="61" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H14" s="66">
+        <f>'Profit Simulation'!H14*$G14</f>
+        <v/>
+      </c>
+      <c r="I14" s="66">
+        <f>'Profit Simulation'!I14*$G14</f>
+        <v/>
+      </c>
+      <c r="J14" s="66">
+        <f>'Profit Simulation'!J14*$G14</f>
+        <v/>
+      </c>
+      <c r="K14" s="66">
+        <f>'Profit Simulation'!K14*$G14</f>
+        <v/>
+      </c>
+      <c r="L14" s="66">
+        <f>'Profit Simulation'!L14*$G14</f>
+        <v/>
+      </c>
+      <c r="M14" s="66">
+        <f>'Profit Simulation'!M14*$G14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TOTAL COMP — Portfolio Manager 1</t>
+        </is>
+      </c>
+      <c r="H15" s="54">
+        <f>SUM(H12:H14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="54">
+        <f>SUM(I12:I14)</f>
+        <v/>
+      </c>
+      <c r="J15" s="54">
+        <f>SUM(J12:J14)</f>
+        <v/>
+      </c>
+      <c r="K15" s="54">
+        <f>SUM(K12:K14)</f>
+        <v/>
+      </c>
+      <c r="L15" s="54">
+        <f>SUM(L12:L14)</f>
+        <v/>
+      </c>
+      <c r="M15" s="54">
+        <f>SUM(M12:M14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="64" t="inlineStr">
+        <is>
+          <t>Portfolio Manager 2  (wt 8, equity 10.0%)</t>
+        </is>
+      </c>
+      <c r="H17" s="65" t="inlineStr"/>
+      <c r="I17" s="65" t="inlineStr"/>
+      <c r="J17" s="65" t="inlineStr"/>
+      <c r="K17" s="65" t="inlineStr"/>
+      <c r="L17" s="65" t="inlineStr"/>
+      <c r="M17" s="65" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Base salary</t>
+        </is>
+      </c>
+      <c r="H18" s="51">
+        <f>IF(Static!H15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+      <c r="I18" s="51">
+        <f>IF(Static!I15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+      <c r="J18" s="51">
+        <f>IF(Static!J15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+      <c r="K18" s="51">
+        <f>IF(Static!K15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+      <c r="L18" s="51">
+        <f>IF(Static!L15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+      <c r="M18" s="51">
+        <f>IF(Static!M15&lt;Static!$F$9,Static!$B$22,Static!$C$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Performance take  (weight × unit value)</t>
+        </is>
+      </c>
+      <c r="H19" s="51">
+        <f>Static!$D$22*Static!H$35</f>
+        <v/>
+      </c>
+      <c r="I19" s="51">
+        <f>Static!$D$22*Static!I$35</f>
+        <v/>
+      </c>
+      <c r="J19" s="51">
+        <f>Static!$D$22*Static!J$35</f>
+        <v/>
+      </c>
+      <c r="K19" s="51">
+        <f>Static!$D$22*Static!K$35</f>
+        <v/>
+      </c>
+      <c r="L19" s="51">
+        <f>Static!$D$22*Static!L$35</f>
+        <v/>
+      </c>
+      <c r="M19" s="51">
+        <f>Static!$D$22*Static!M$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Equity distribution  (10.0% × EBIT)</t>
+        </is>
+      </c>
+      <c r="G20" s="61" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H20" s="66">
+        <f>'Profit Simulation'!H14*$G20</f>
+        <v/>
+      </c>
+      <c r="I20" s="66">
+        <f>'Profit Simulation'!I14*$G20</f>
+        <v/>
+      </c>
+      <c r="J20" s="66">
+        <f>'Profit Simulation'!J14*$G20</f>
+        <v/>
+      </c>
+      <c r="K20" s="66">
+        <f>'Profit Simulation'!K14*$G20</f>
+        <v/>
+      </c>
+      <c r="L20" s="66">
+        <f>'Profit Simulation'!L14*$G20</f>
+        <v/>
+      </c>
+      <c r="M20" s="66">
+        <f>'Profit Simulation'!M14*$G20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TOTAL COMP — Portfolio Manager 2</t>
+        </is>
+      </c>
+      <c r="H21" s="54">
+        <f>SUM(H18:H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="54">
+        <f>SUM(I18:I20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="54">
+        <f>SUM(J18:J20)</f>
+        <v/>
+      </c>
+      <c r="K21" s="54">
+        <f>SUM(K18:K20)</f>
+        <v/>
+      </c>
+      <c r="L21" s="54">
+        <f>SUM(L18:L20)</f>
+        <v/>
+      </c>
+      <c r="M21" s="54">
+        <f>SUM(M18:M20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="67" t="inlineStr">
+        <is>
+          <t>Both PMs combined (equity 20%)</t>
+        </is>
+      </c>
+      <c r="H23" s="68">
+        <f>H13*2</f>
+        <v/>
+      </c>
+      <c r="I23" s="68">
+        <f>I13*2</f>
+        <v/>
+      </c>
+      <c r="J23" s="68">
+        <f>J13*2</f>
+        <v/>
+      </c>
+      <c r="K23" s="68">
+        <f>K13*2</f>
+        <v/>
+      </c>
+      <c r="L23" s="68">
+        <f>L13*2</f>
+        <v/>
+      </c>
+      <c r="M23" s="68">
+        <f>M13*2</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>